<commit_message>
Update ODCS template files and examples with v3.2 changes
</commit_message>
<xml_diff>
--- a/examples/full-odcs-3.2.xlsx
+++ b/examples/full-odcs-3.2.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema orders" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema shipments" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema shipments_archive" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servers" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Authoritative Definitions" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified Statements" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constraints" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enums" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synonyms" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Properties" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ServerFields" sheetId="20" state="hidden" r:id="rId20"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schema orders" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Schema shipments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Schema shipments_archive" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Relationships" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Quality" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Support" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Team" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Roles" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SLA" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Servers" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Pricing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Authoritative Definitions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Verified Statements" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Constraints" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Enums" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Synonyms" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Custom Properties" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="_ServerFields" sheetId="20" state="hidden" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_ServerFieldLabels">_ServerFields!$A$2:$A$24</definedName>
@@ -34,20 +34,20 @@
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
     <definedName name="authoritativeDefinitions">'Authoritative Definitions'!$A$4:$F$1000</definedName>
     <definedName name="constraints">Constraints!$A$4:$AZ$1000</definedName>
-    <definedName name="context.instructions">Fundamentals!$C$25</definedName>
-    <definedName name="CustomProperties">'Custom Properties'!$A$5:$G$21</definedName>
+    <definedName name="context.instructions">Fundamentals!$C$26</definedName>
+    <definedName name="CustomProperties">'Custom Properties'!$A$5:$H$21</definedName>
     <definedName name="datacontract_id">Fundamentals!$C$7</definedName>
-    <definedName name="dataProduct">Fundamentals!$C$15</definedName>
-    <definedName name="description.limitations">Fundamentals!$C$20</definedName>
-    <definedName name="description.purpose">Fundamentals!$C$19</definedName>
-    <definedName name="description.usage">Fundamentals!$C$21</definedName>
-    <definedName name="domain">Fundamentals!$C$14</definedName>
+    <definedName name="dataProduct">Fundamentals!$C$16</definedName>
+    <definedName name="description.limitations">Fundamentals!$C$21</definedName>
+    <definedName name="description.purpose">Fundamentals!$C$20</definedName>
+    <definedName name="description.usage">Fundamentals!$C$22</definedName>
+    <definedName name="domain">Fundamentals!$C$15</definedName>
     <definedName name="enum">Enums!$A$4:$AZ$1000</definedName>
     <definedName name="id">Fundamentals!$C$7</definedName>
     <definedName name="instructions.importUrl">Instructions!$B$24</definedName>
     <definedName name="kind">Fundamentals!$C$4</definedName>
     <definedName name="name">Fundamentals!$C$8</definedName>
-    <definedName name="owner">Fundamentals!$C$12</definedName>
+    <definedName name="owner">Fundamentals!$C$13</definedName>
     <definedName name="price.id">Pricing!$B$7</definedName>
     <definedName name="price.priceAmount">Pricing!$B$4</definedName>
     <definedName name="price.priceCurrency">Pricing!$B$5</definedName>
@@ -86,17 +86,16 @@
     <definedName name="status">Fundamentals!$C$10</definedName>
     <definedName name="support">Support!$A$4:$AZ$1000</definedName>
     <definedName name="synonyms">Synonyms!$A$4:$AZ$1000</definedName>
-    <definedName name="tags">Fundamentals!$C$23</definedName>
-    <definedName name="team">Team!$A$10:$AZ$1006</definedName>
+    <definedName name="tags">Fundamentals!$C$24</definedName>
+    <definedName name="team">Team!$A$10:$BA$1006</definedName>
     <definedName name="team.description">Team!$B$5</definedName>
     <definedName name="team.id">Team!$B$7</definedName>
     <definedName name="team.name">Team!$B$4</definedName>
     <definedName name="team.tags">Team!$B$6</definedName>
-    <definedName name="tenant">Fundamentals!$C$16</definedName>
+    <definedName name="tenant">Fundamentals!$C$17</definedName>
     <definedName name="verifiedStatements">'Verified Statements'!$A$4:$AZ$1000</definedName>
     <definedName name="version">Fundamentals!$C$9</definedName>
-    <definedName name="roles" localSheetId="9">Roles!$A$4:$AZ$1000</definedName>
-    <definedName name="slaProperties" localSheetId="10">SLA!$A$6:$AZ$1002</definedName>
+    <definedName name="contractCreatedTs">Fundamentals!$C$11</definedName>
     <definedName name="schema.businessName" localSheetId="2">'Schema orders'!$B$8</definedName>
     <definedName name="schema.context.instructions" localSheetId="2">'Schema orders'!$B$13</definedName>
     <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema orders'!$B$10</definedName>
@@ -106,7 +105,7 @@
     <definedName name="schema.name" localSheetId="2">'Schema orders'!$B$5</definedName>
     <definedName name="schema.physicalName" localSheetId="2">'Schema orders'!$B$9</definedName>
     <definedName name="schema.physicalType" localSheetId="2">'Schema orders'!$B$6</definedName>
-    <definedName name="schema.properties" localSheetId="2">'Schema orders'!$A$16:$AO$984</definedName>
+    <definedName name="schema.properties" localSheetId="2">'Schema orders'!$A$16:$AW$984</definedName>
     <definedName name="schema.tags" localSheetId="2">'Schema orders'!$B$11</definedName>
     <definedName name="schema.businessName" localSheetId="3">'Schema shipments'!$B$8</definedName>
     <definedName name="schema.context.instructions" localSheetId="3">'Schema shipments'!$B$13</definedName>
@@ -117,7 +116,7 @@
     <definedName name="schema.name" localSheetId="3">'Schema shipments'!$B$5</definedName>
     <definedName name="schema.physicalName" localSheetId="3">'Schema shipments'!$B$9</definedName>
     <definedName name="schema.physicalType" localSheetId="3">'Schema shipments'!$B$6</definedName>
-    <definedName name="schema.properties" localSheetId="3">'Schema shipments'!$A$16:$AO$984</definedName>
+    <definedName name="schema.properties" localSheetId="3">'Schema shipments'!$A$16:$AW$984</definedName>
     <definedName name="schema.tags" localSheetId="3">'Schema shipments'!$B$11</definedName>
     <definedName name="schema.businessName" localSheetId="4">'Schema shipments_archive'!$B$8</definedName>
     <definedName name="schema.context.instructions" localSheetId="4">'Schema shipments_archive'!$B$13</definedName>
@@ -128,8 +127,10 @@
     <definedName name="schema.name" localSheetId="4">'Schema shipments_archive'!$B$5</definedName>
     <definedName name="schema.physicalName" localSheetId="4">'Schema shipments_archive'!$B$9</definedName>
     <definedName name="schema.physicalType" localSheetId="4">'Schema shipments_archive'!$B$6</definedName>
-    <definedName name="schema.properties" localSheetId="4">'Schema shipments_archive'!$A$16:$AO$984</definedName>
+    <definedName name="schema.properties" localSheetId="4">'Schema shipments_archive'!$A$16:$AW$984</definedName>
     <definedName name="schema.tags" localSheetId="4">'Schema shipments_archive'!$B$11</definedName>
+    <definedName name="roles" localSheetId="9">Roles!$A$4:$AZ$1000</definedName>
+    <definedName name="slaProperties" localSheetId="10">SLA!$A$6:$AZ$1002</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -15465,7 +15466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="19.6640625" customWidth="1" style="2" min="1" max="1"/>
@@ -15520,17 +15521,22 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Value Type</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -15552,9 +15558,9 @@
         <f>IF(owner &lt;&gt; "", owner, "")</f>
         <v/>
       </c>
-      <c r="E5" s="36" t="n"/>
       <c r="F5" s="36" t="n"/>
       <c r="G5" s="36" t="n"/>
+      <c r="H5" s="36" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="36" t="inlineStr">
@@ -15571,17 +15577,17 @@
       <c r="D6" s="36" t="n">
         <v>730</v>
       </c>
-      <c r="E6" s="36" t="inlineStr">
+      <c r="F6" s="36" t="inlineStr">
         <is>
           <t>How long rows are kept before they move to the archive.</t>
         </is>
       </c>
-      <c r="F6" s="36" t="inlineStr">
+      <c r="G6" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G6" s="36" t="inlineStr">
+      <c r="H6" s="36" t="inlineStr">
         <is>
           <t>retentionDays</t>
         </is>
@@ -15604,17 +15610,17 @@
           <t>docs-team</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="F7" s="36" t="inlineStr">
         <is>
           <t>Who maintains the description block.</t>
         </is>
       </c>
-      <c r="F7" s="36" t="inlineStr">
+      <c r="G7" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G7" s="36" t="inlineStr">
+      <c r="H7" s="36" t="inlineStr">
         <is>
           <t>descriptionOwnerProp</t>
         </is>
@@ -15641,17 +15647,17 @@
           <t>analytics-guild</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="F8" s="36" t="inlineStr">
         <is>
           <t>Who verified the answer.</t>
         </is>
       </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="G8" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G8" s="36" t="inlineStr">
+      <c r="H8" s="36" t="inlineStr">
         <is>
           <t>verifiedStatementReviewer</t>
         </is>
@@ -15678,17 +15684,17 @@
           <t>policy-engine</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="F9" s="36" t="inlineStr">
         <is>
           <t>System enforcing the constraint.</t>
         </is>
       </c>
-      <c r="F9" s="36" t="inlineStr">
+      <c r="G9" s="36" t="inlineStr">
         <is>
           <t>opa</t>
         </is>
       </c>
-      <c r="G9" s="36" t="inlineStr">
+      <c r="H9" s="36" t="inlineStr">
         <is>
           <t>constraintEnforcer</t>
         </is>
@@ -15715,17 +15721,17 @@
           <t>entitlement-service</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="F10" s="36" t="inlineStr">
         <is>
           <t>How the role is granted.</t>
         </is>
       </c>
-      <c r="F10" s="36" t="inlineStr">
+      <c r="G10" s="36" t="inlineStr">
         <is>
           <t>sailpoint</t>
         </is>
       </c>
-      <c r="G10" s="36" t="inlineStr">
+      <c r="H10" s="36" t="inlineStr">
         <is>
           <t>analystRoleGrant</t>
         </is>
@@ -15752,17 +15758,17 @@
           <t>iam</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="F11" s="36" t="inlineStr">
         <is>
           <t>How server access is granted.</t>
         </is>
       </c>
-      <c r="F11" s="36" t="inlineStr">
+      <c r="G11" s="36" t="inlineStr">
         <is>
           <t>aws</t>
         </is>
       </c>
-      <c r="G11" s="36" t="inlineStr">
+      <c r="H11" s="36" t="inlineStr">
         <is>
           <t>serverRoleGrant</t>
         </is>
@@ -15789,17 +15795,17 @@
           <t>CC-4711</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="F12" s="36" t="inlineStr">
         <is>
           <t>Cost center the team bills to.</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>sap</t>
         </is>
       </c>
-      <c r="G12" s="36" t="inlineStr">
+      <c r="H12" s="36" t="inlineStr">
         <is>
           <t>teamCostCenter</t>
         </is>
@@ -15826,17 +15832,17 @@
           <t>@jdoe</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="F13" s="36" t="inlineStr">
         <is>
           <t>Slack handle of the member.</t>
         </is>
       </c>
-      <c r="F13" s="36" t="inlineStr">
+      <c r="G13" s="36" t="inlineStr">
         <is>
           <t>slack</t>
         </is>
       </c>
-      <c r="G13" s="36" t="inlineStr">
+      <c r="H13" s="36" t="inlineStr">
         <is>
           <t>memberJdoeSlack</t>
         </is>
@@ -15861,17 +15867,17 @@
       <c r="D14" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="36" t="inlineStr">
+      <c r="F14" s="36" t="inlineStr">
         <is>
           <t>Target first response time.</t>
         </is>
       </c>
-      <c r="F14" s="36" t="inlineStr">
+      <c r="G14" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G14" s="36" t="inlineStr">
+      <c r="H14" s="36" t="inlineStr">
         <is>
           <t>supportResponseTime</t>
         </is>
@@ -15898,17 +15904,17 @@
           <t>soda-cloud-monitor</t>
         </is>
       </c>
-      <c r="E15" s="36" t="inlineStr">
+      <c r="F15" s="36" t="inlineStr">
         <is>
           <t>Monitor producing the measurement.</t>
         </is>
       </c>
-      <c r="F15" s="36" t="inlineStr">
+      <c r="G15" s="36" t="inlineStr">
         <is>
           <t>soda</t>
         </is>
       </c>
-      <c r="G15" s="36" t="inlineStr">
+      <c r="H15" s="36" t="inlineStr">
         <is>
           <t>slaLatencyMonitor</t>
         </is>
@@ -15935,17 +15941,17 @@
           <t>dmz</t>
         </is>
       </c>
-      <c r="E16" s="36" t="inlineStr">
+      <c r="F16" s="36" t="inlineStr">
         <is>
           <t>Network zone of the server.</t>
         </is>
       </c>
-      <c r="F16" s="36" t="inlineStr">
+      <c r="G16" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G16" s="36" t="inlineStr">
+      <c r="H16" s="36" t="inlineStr">
         <is>
           <t>serverNetworkZone</t>
         </is>
@@ -15972,17 +15978,17 @@
           <t>erp</t>
         </is>
       </c>
-      <c r="E17" s="36" t="inlineStr">
+      <c r="F17" s="36" t="inlineStr">
         <is>
           <t>System of record.</t>
         </is>
       </c>
-      <c r="F17" s="36" t="inlineStr">
+      <c r="G17" s="36" t="inlineStr">
         <is>
           <t>sap</t>
         </is>
       </c>
-      <c r="G17" s="36" t="inlineStr">
+      <c r="H17" s="36" t="inlineStr">
         <is>
           <t>ordersSourceSystem</t>
         </is>
@@ -16009,17 +16015,17 @@
           <t>hourly</t>
         </is>
       </c>
-      <c r="E18" s="36" t="inlineStr">
+      <c r="F18" s="36" t="inlineStr">
         <is>
           <t>How often the table is refreshed.</t>
         </is>
       </c>
-      <c r="F18" s="36" t="inlineStr">
+      <c r="G18" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G18" s="36" t="inlineStr">
+      <c r="H18" s="36" t="inlineStr">
         <is>
           <t>shipmentsRefreshCadence</t>
         </is>
@@ -16046,17 +16052,17 @@
           <t>data-governance</t>
         </is>
       </c>
-      <c r="E19" s="36" t="inlineStr">
+      <c r="F19" s="36" t="inlineStr">
         <is>
           <t>Who approved the synonym.</t>
         </is>
       </c>
-      <c r="F19" s="36" t="inlineStr">
+      <c r="G19" s="36" t="inlineStr">
         <is>
           <t>collibra</t>
         </is>
       </c>
-      <c r="G19" s="36" t="inlineStr">
+      <c r="H19" s="36" t="inlineStr">
         <is>
           <t>ordersSynonymApproval</t>
         </is>
@@ -16083,17 +16089,17 @@
           <t>2024-01-01</t>
         </is>
       </c>
-      <c r="E20" s="36" t="inlineStr">
+      <c r="F20" s="36" t="inlineStr">
         <is>
           <t>When the synonym was retired.</t>
         </is>
       </c>
-      <c r="F20" s="36" t="inlineStr">
+      <c r="G20" s="36" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G20" s="36" t="inlineStr">
+      <c r="H20" s="36" t="inlineStr">
         <is>
           <t>shipmentIdSynonymRetired</t>
         </is>
@@ -16120,17 +16126,17 @@
           <t>airflow</t>
         </is>
       </c>
-      <c r="E21" s="36" t="inlineStr">
+      <c r="F21" s="36" t="inlineStr">
         <is>
           <t>Orchestrator running the check.</t>
         </is>
       </c>
-      <c r="F21" s="36" t="inlineStr">
+      <c r="G21" s="36" t="inlineStr">
         <is>
           <t>airflow</t>
         </is>
       </c>
-      <c r="G21" s="36" t="inlineStr">
+      <c r="H21" s="36" t="inlineStr">
         <is>
           <t>ordersRowCountRunner</t>
         </is>
@@ -16157,17 +16163,17 @@
           <t>airflow</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Orchestrator running the check.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>airflow</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>shipmentIdUniqueRunner</t>
         </is>
@@ -16194,17 +16200,17 @@
           <t>mask_uuid</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Masking policy applied in the warehouse.</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>snowflake</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>shipmentIdMasking</t>
         </is>
@@ -16233,15 +16239,20 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>Whether the database enforces the key.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>orderFkEnforced</t>
         </is>
@@ -16270,15 +16281,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>Whether the database enforces the key.</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>compositeKeyEnforced</t>
         </is>
@@ -16305,17 +16321,17 @@
           <t>FedEx</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>German label.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>carrierFedexLabelDe</t>
         </is>
@@ -16342,17 +16358,17 @@
           <t>analytics-guild</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Who verified the answer.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>entropy-data</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>shipmentsStatementReviewer</t>
         </is>
@@ -16379,17 +16395,17 @@
           <t>policy-engine</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>System enforcing the constraint.</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>opa</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>shipmentsConstraintEnforcer</t>
         </is>
@@ -16412,7 +16428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="2.83203125" customWidth="1" style="2" min="1" max="1"/>
@@ -16526,51 +16542,48 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="34" t="n"/>
-      <c r="B11" s="34" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Contract Created</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-01-15T09:00:00Z</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="34" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="B12" s="40" t="n"/>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="B13" s="40" t="n"/>
+      <c r="C13" s="36" t="inlineStr">
         <is>
           <t>logistics-platform-team</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="34" t="n"/>
-      <c r="B13" s="34" t="n"/>
+      <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
+      <c r="A14" s="34" t="n"/>
       <c r="B14" s="34" t="n"/>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
-          <t>logistics</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="34" t="inlineStr">
         <is>
-          <t>Data Product</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B15" s="34" t="n"/>
       <c r="C15" s="36" t="inlineStr">
         <is>
-          <t>shipment-analytics</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
@@ -16578,51 +16591,52 @@
     <row r="16">
       <c r="A16" s="34" t="inlineStr">
         <is>
-          <t>Tenant</t>
+          <t>Data Product</t>
         </is>
       </c>
       <c r="B16" s="34" t="n"/>
       <c r="C16" s="36" t="inlineStr">
         <is>
+          <t>shipment-analytics</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>Tenant</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="n"/>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
           <t>acme-eu</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="34" t="n"/>
-      <c r="B17" s="34" t="n"/>
-    </row>
     <row r="18">
-      <c r="A18" s="34" t="inlineStr">
+      <c r="A18" s="34" t="n"/>
+      <c r="B18" s="34" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B18" s="34" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="34" t="n"/>
-      <c r="B19" s="34" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="C19" s="36" t="inlineStr">
-        <is>
-          <t>Analytical view of parcel shipments, used for delivery performance reporting. Demonstrates every element of ODCS v3.2.0.</t>
-        </is>
-      </c>
+      <c r="B19" s="34" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="34" t="n"/>
       <c r="B20" s="34" t="inlineStr">
         <is>
-          <t>Limitations</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="C20" s="36" t="inlineStr">
         <is>
-          <t>Illustrative example data, not a production data set.</t>
+          <t>Analytical view of parcel shipments, used for delivery performance reporting. Demonstrates every element of ODCS v3.2.0.</t>
         </is>
       </c>
     </row>
@@ -16630,46 +16644,59 @@
       <c r="A21" s="34" t="n"/>
       <c r="B21" s="34" t="inlineStr">
         <is>
-          <t>Usage</t>
+          <t>Limitations</t>
         </is>
       </c>
       <c r="C21" s="36" t="inlineStr">
         <is>
-          <t>Use as a reference when authoring a data contract or filling in the Excel template.</t>
+          <t>Illustrative example data, not a production data set.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="34" t="n"/>
-      <c r="B22" s="34" t="n"/>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>Usage</t>
+        </is>
+      </c>
+      <c r="C22" s="36" t="inlineStr">
+        <is>
+          <t>Use as a reference when authoring a data contract or filling in the Excel template.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="34" t="inlineStr">
+      <c r="A23" s="34" t="n"/>
+      <c r="B23" s="34" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="B23" s="34" t="n"/>
-      <c r="C23" s="36" t="inlineStr">
-        <is>
-          <t>coverage,datalocation:EU</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="34" t="inlineStr">
+      <c r="B24" s="34" t="n"/>
+      <c r="C24" s="36" t="inlineStr">
+        <is>
+          <t>logistics,datalocation:EU</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="34" t="inlineStr">
         <is>
           <t>Context Instructions</t>
         </is>
       </c>
-      <c r="C25" s="36" t="inlineStr">
+      <c r="C26" s="36" t="inlineStr">
         <is>
           <t>One row in shipments is one physical parcel. Join to orders through order_id. All timestamps are UTC.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="2" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>as Guidance for AI</t>
         </is>
@@ -17932,7 +17959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR52"/>
+  <dimension ref="A1:AZ52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="34.83203125" customWidth="1" style="2" min="1" max="1"/>
@@ -18149,13 +18176,13 @@
       <c r="AK15" s="20" t="n"/>
       <c r="AL15" s="20" t="n"/>
       <c r="AM15" s="21" t="n"/>
-      <c r="AP15" s="19" t="inlineStr">
+      <c r="AX15" s="19" t="inlineStr">
         <is>
           <t>Custom Properties</t>
         </is>
       </c>
-      <c r="AQ15" s="20" t="n"/>
-      <c r="AR15" s="20" t="n"/>
+      <c r="AY15" s="20" t="n"/>
+      <c r="AZ15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -18353,19 +18380,59 @@
           <t>Pattern</t>
         </is>
       </c>
-      <c r="AN16" s="10" t="inlineStr">
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>Element Type</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Distance Metric</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Normalized</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>Embedding Model</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>Embedding Model Version</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Default Timezone</t>
+        </is>
+      </c>
+      <c r="AV16" s="10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="AO16" s="10" t="inlineStr">
+      <c r="AW16" s="10" t="inlineStr">
         <is>
           <t>Comments (internal)</t>
         </is>
       </c>
-      <c r="AP16" s="10" t="n"/>
-      <c r="AQ16" s="10" t="n"/>
-      <c r="AR16" s="10" t="n"/>
+      <c r="AX16" s="10" t="n"/>
+      <c r="AY16" s="10" t="n"/>
+      <c r="AZ16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -18425,15 +18492,15 @@
       <c r="AK17" s="15" t="n"/>
       <c r="AL17" s="15" t="n"/>
       <c r="AM17" s="15" t="n"/>
-      <c r="AN17" s="15" t="inlineStr">
+      <c r="AV17" s="15" t="inlineStr">
         <is>
           <t>ordersOrderId</t>
         </is>
       </c>
-      <c r="AO17" s="28" t="n"/>
-      <c r="AP17" s="15" t="n"/>
-      <c r="AQ17" s="15" t="n"/>
-      <c r="AR17" s="15" t="n"/>
+      <c r="AW17" s="28" t="n"/>
+      <c r="AX17" s="15" t="n"/>
+      <c r="AY17" s="15" t="n"/>
+      <c r="AZ17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -18491,15 +18558,15 @@
       <c r="AK18" s="15" t="n"/>
       <c r="AL18" s="15" t="n"/>
       <c r="AM18" s="15" t="n"/>
-      <c r="AN18" s="15" t="inlineStr">
+      <c r="AV18" s="15" t="inlineStr">
         <is>
           <t>ordersCarrierCode</t>
         </is>
       </c>
-      <c r="AO18" s="28" t="n"/>
-      <c r="AP18" s="15" t="n"/>
-      <c r="AQ18" s="15" t="n"/>
-      <c r="AR18" s="15" t="n"/>
+      <c r="AW18" s="28" t="n"/>
+      <c r="AX18" s="15" t="n"/>
+      <c r="AY18" s="15" t="n"/>
+      <c r="AZ18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -18553,11 +18620,11 @@
       <c r="AK19" s="15" t="n"/>
       <c r="AL19" s="15" t="n"/>
       <c r="AM19" s="15" t="n"/>
-      <c r="AN19" s="15" t="n"/>
-      <c r="AO19" s="28" t="n"/>
-      <c r="AP19" s="15" t="n"/>
-      <c r="AQ19" s="15" t="n"/>
-      <c r="AR19" s="15" t="n"/>
+      <c r="AV19" s="15" t="n"/>
+      <c r="AW19" s="28" t="n"/>
+      <c r="AX19" s="15" t="n"/>
+      <c r="AY19" s="15" t="n"/>
+      <c r="AZ19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="17" t="n"/>
@@ -18599,11 +18666,11 @@
       <c r="AK20" s="15" t="n"/>
       <c r="AL20" s="15" t="n"/>
       <c r="AM20" s="15" t="n"/>
-      <c r="AN20" s="15" t="n"/>
-      <c r="AO20" s="28" t="n"/>
-      <c r="AP20" s="15" t="n"/>
-      <c r="AQ20" s="15" t="n"/>
-      <c r="AR20" s="15" t="n"/>
+      <c r="AV20" s="15" t="n"/>
+      <c r="AW20" s="28" t="n"/>
+      <c r="AX20" s="15" t="n"/>
+      <c r="AY20" s="15" t="n"/>
+      <c r="AZ20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="17" t="n"/>
@@ -18645,11 +18712,11 @@
       <c r="AK21" s="15" t="n"/>
       <c r="AL21" s="15" t="n"/>
       <c r="AM21" s="15" t="n"/>
-      <c r="AN21" s="15" t="n"/>
-      <c r="AO21" s="28" t="n"/>
-      <c r="AP21" s="15" t="n"/>
-      <c r="AQ21" s="15" t="n"/>
-      <c r="AR21" s="15" t="n"/>
+      <c r="AV21" s="15" t="n"/>
+      <c r="AW21" s="28" t="n"/>
+      <c r="AX21" s="15" t="n"/>
+      <c r="AY21" s="15" t="n"/>
+      <c r="AZ21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="17" t="n"/>
@@ -18691,11 +18758,11 @@
       <c r="AK22" s="15" t="n"/>
       <c r="AL22" s="15" t="n"/>
       <c r="AM22" s="15" t="n"/>
-      <c r="AN22" s="15" t="n"/>
-      <c r="AO22" s="28" t="n"/>
-      <c r="AP22" s="15" t="n"/>
-      <c r="AQ22" s="15" t="n"/>
-      <c r="AR22" s="15" t="n"/>
+      <c r="AV22" s="15" t="n"/>
+      <c r="AW22" s="28" t="n"/>
+      <c r="AX22" s="15" t="n"/>
+      <c r="AY22" s="15" t="n"/>
+      <c r="AZ22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="17" t="n"/>
@@ -18737,11 +18804,11 @@
       <c r="AK23" s="15" t="n"/>
       <c r="AL23" s="15" t="n"/>
       <c r="AM23" s="15" t="n"/>
-      <c r="AN23" s="15" t="n"/>
-      <c r="AO23" s="28" t="n"/>
-      <c r="AP23" s="15" t="n"/>
-      <c r="AQ23" s="15" t="n"/>
-      <c r="AR23" s="15" t="n"/>
+      <c r="AV23" s="15" t="n"/>
+      <c r="AW23" s="28" t="n"/>
+      <c r="AX23" s="15" t="n"/>
+      <c r="AY23" s="15" t="n"/>
+      <c r="AZ23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="n"/>
@@ -18783,11 +18850,11 @@
       <c r="AK24" s="15" t="n"/>
       <c r="AL24" s="15" t="n"/>
       <c r="AM24" s="15" t="n"/>
-      <c r="AN24" s="15" t="n"/>
-      <c r="AO24" s="28" t="n"/>
-      <c r="AP24" s="15" t="n"/>
-      <c r="AQ24" s="15" t="n"/>
-      <c r="AR24" s="15" t="n"/>
+      <c r="AV24" s="15" t="n"/>
+      <c r="AW24" s="28" t="n"/>
+      <c r="AX24" s="15" t="n"/>
+      <c r="AY24" s="15" t="n"/>
+      <c r="AZ24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="18" t="n"/>
@@ -18829,11 +18896,11 @@
       <c r="AK25" s="15" t="n"/>
       <c r="AL25" s="15" t="n"/>
       <c r="AM25" s="15" t="n"/>
-      <c r="AN25" s="15" t="n"/>
-      <c r="AO25" s="28" t="n"/>
-      <c r="AP25" s="15" t="n"/>
-      <c r="AQ25" s="15" t="n"/>
-      <c r="AR25" s="15" t="n"/>
+      <c r="AV25" s="15" t="n"/>
+      <c r="AW25" s="28" t="n"/>
+      <c r="AX25" s="15" t="n"/>
+      <c r="AY25" s="15" t="n"/>
+      <c r="AZ25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="18" t="n"/>
@@ -18875,11 +18942,11 @@
       <c r="AK26" s="15" t="n"/>
       <c r="AL26" s="15" t="n"/>
       <c r="AM26" s="15" t="n"/>
-      <c r="AN26" s="15" t="n"/>
-      <c r="AO26" s="28" t="n"/>
-      <c r="AP26" s="15" t="n"/>
-      <c r="AQ26" s="15" t="n"/>
-      <c r="AR26" s="15" t="n"/>
+      <c r="AV26" s="15" t="n"/>
+      <c r="AW26" s="28" t="n"/>
+      <c r="AX26" s="15" t="n"/>
+      <c r="AY26" s="15" t="n"/>
+      <c r="AZ26" s="15" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="17" t="n"/>
@@ -18921,11 +18988,11 @@
       <c r="AK27" s="15" t="n"/>
       <c r="AL27" s="15" t="n"/>
       <c r="AM27" s="15" t="n"/>
-      <c r="AN27" s="15" t="n"/>
-      <c r="AO27" s="28" t="n"/>
-      <c r="AP27" s="15" t="n"/>
-      <c r="AQ27" s="15" t="n"/>
-      <c r="AR27" s="15" t="n"/>
+      <c r="AV27" s="15" t="n"/>
+      <c r="AW27" s="28" t="n"/>
+      <c r="AX27" s="15" t="n"/>
+      <c r="AY27" s="15" t="n"/>
+      <c r="AZ27" s="15" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="17" t="n"/>
@@ -18967,11 +19034,11 @@
       <c r="AK28" s="15" t="n"/>
       <c r="AL28" s="15" t="n"/>
       <c r="AM28" s="15" t="n"/>
-      <c r="AN28" s="15" t="n"/>
-      <c r="AO28" s="28" t="n"/>
-      <c r="AP28" s="15" t="n"/>
-      <c r="AQ28" s="15" t="n"/>
-      <c r="AR28" s="15" t="n"/>
+      <c r="AV28" s="15" t="n"/>
+      <c r="AW28" s="28" t="n"/>
+      <c r="AX28" s="15" t="n"/>
+      <c r="AY28" s="15" t="n"/>
+      <c r="AZ28" s="15" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="17" t="n"/>
@@ -19013,11 +19080,11 @@
       <c r="AK29" s="15" t="n"/>
       <c r="AL29" s="15" t="n"/>
       <c r="AM29" s="15" t="n"/>
-      <c r="AN29" s="15" t="n"/>
-      <c r="AO29" s="28" t="n"/>
-      <c r="AP29" s="15" t="n"/>
-      <c r="AQ29" s="15" t="n"/>
-      <c r="AR29" s="15" t="n"/>
+      <c r="AV29" s="15" t="n"/>
+      <c r="AW29" s="28" t="n"/>
+      <c r="AX29" s="15" t="n"/>
+      <c r="AY29" s="15" t="n"/>
+      <c r="AZ29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="17" t="n"/>
@@ -19059,11 +19126,11 @@
       <c r="AK30" s="15" t="n"/>
       <c r="AL30" s="15" t="n"/>
       <c r="AM30" s="15" t="n"/>
-      <c r="AN30" s="15" t="n"/>
-      <c r="AO30" s="28" t="n"/>
-      <c r="AP30" s="15" t="n"/>
-      <c r="AQ30" s="15" t="n"/>
-      <c r="AR30" s="15" t="n"/>
+      <c r="AV30" s="15" t="n"/>
+      <c r="AW30" s="28" t="n"/>
+      <c r="AX30" s="15" t="n"/>
+      <c r="AY30" s="15" t="n"/>
+      <c r="AZ30" s="15" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="n"/>
@@ -19105,11 +19172,11 @@
       <c r="AK31" s="15" t="n"/>
       <c r="AL31" s="15" t="n"/>
       <c r="AM31" s="15" t="n"/>
-      <c r="AN31" s="15" t="n"/>
-      <c r="AO31" s="28" t="n"/>
-      <c r="AP31" s="15" t="n"/>
-      <c r="AQ31" s="15" t="n"/>
-      <c r="AR31" s="15" t="n"/>
+      <c r="AV31" s="15" t="n"/>
+      <c r="AW31" s="28" t="n"/>
+      <c r="AX31" s="15" t="n"/>
+      <c r="AY31" s="15" t="n"/>
+      <c r="AZ31" s="15" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="17" t="n"/>
@@ -19151,11 +19218,11 @@
       <c r="AK32" s="15" t="n"/>
       <c r="AL32" s="15" t="n"/>
       <c r="AM32" s="15" t="n"/>
-      <c r="AN32" s="15" t="n"/>
-      <c r="AO32" s="28" t="n"/>
-      <c r="AP32" s="15" t="n"/>
-      <c r="AQ32" s="15" t="n"/>
-      <c r="AR32" s="15" t="n"/>
+      <c r="AV32" s="15" t="n"/>
+      <c r="AW32" s="28" t="n"/>
+      <c r="AX32" s="15" t="n"/>
+      <c r="AY32" s="15" t="n"/>
+      <c r="AZ32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="n"/>
@@ -19197,11 +19264,11 @@
       <c r="AK33" s="15" t="n"/>
       <c r="AL33" s="15" t="n"/>
       <c r="AM33" s="15" t="n"/>
-      <c r="AN33" s="15" t="n"/>
-      <c r="AO33" s="28" t="n"/>
-      <c r="AP33" s="15" t="n"/>
-      <c r="AQ33" s="15" t="n"/>
-      <c r="AR33" s="15" t="n"/>
+      <c r="AV33" s="15" t="n"/>
+      <c r="AW33" s="28" t="n"/>
+      <c r="AX33" s="15" t="n"/>
+      <c r="AY33" s="15" t="n"/>
+      <c r="AZ33" s="15" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="17" t="n"/>
@@ -19243,11 +19310,11 @@
       <c r="AK34" s="15" t="n"/>
       <c r="AL34" s="15" t="n"/>
       <c r="AM34" s="15" t="n"/>
-      <c r="AN34" s="15" t="n"/>
-      <c r="AO34" s="28" t="n"/>
-      <c r="AP34" s="15" t="n"/>
-      <c r="AQ34" s="15" t="n"/>
-      <c r="AR34" s="15" t="n"/>
+      <c r="AV34" s="15" t="n"/>
+      <c r="AW34" s="28" t="n"/>
+      <c r="AX34" s="15" t="n"/>
+      <c r="AY34" s="15" t="n"/>
+      <c r="AZ34" s="15" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="17" t="n"/>
@@ -19289,11 +19356,11 @@
       <c r="AK35" s="15" t="n"/>
       <c r="AL35" s="15" t="n"/>
       <c r="AM35" s="15" t="n"/>
-      <c r="AN35" s="15" t="n"/>
-      <c r="AO35" s="28" t="n"/>
-      <c r="AP35" s="15" t="n"/>
-      <c r="AQ35" s="15" t="n"/>
-      <c r="AR35" s="15" t="n"/>
+      <c r="AV35" s="15" t="n"/>
+      <c r="AW35" s="28" t="n"/>
+      <c r="AX35" s="15" t="n"/>
+      <c r="AY35" s="15" t="n"/>
+      <c r="AZ35" s="15" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="17" t="n"/>
@@ -19335,11 +19402,11 @@
       <c r="AK36" s="15" t="n"/>
       <c r="AL36" s="15" t="n"/>
       <c r="AM36" s="15" t="n"/>
-      <c r="AN36" s="15" t="n"/>
-      <c r="AO36" s="28" t="n"/>
-      <c r="AP36" s="15" t="n"/>
-      <c r="AQ36" s="15" t="n"/>
-      <c r="AR36" s="15" t="n"/>
+      <c r="AV36" s="15" t="n"/>
+      <c r="AW36" s="28" t="n"/>
+      <c r="AX36" s="15" t="n"/>
+      <c r="AY36" s="15" t="n"/>
+      <c r="AZ36" s="15" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="17" t="n"/>
@@ -19381,11 +19448,11 @@
       <c r="AK37" s="15" t="n"/>
       <c r="AL37" s="15" t="n"/>
       <c r="AM37" s="15" t="n"/>
-      <c r="AN37" s="15" t="n"/>
-      <c r="AO37" s="28" t="n"/>
-      <c r="AP37" s="15" t="n"/>
-      <c r="AQ37" s="15" t="n"/>
-      <c r="AR37" s="15" t="n"/>
+      <c r="AV37" s="15" t="n"/>
+      <c r="AW37" s="28" t="n"/>
+      <c r="AX37" s="15" t="n"/>
+      <c r="AY37" s="15" t="n"/>
+      <c r="AZ37" s="15" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="17" t="n"/>
@@ -19427,11 +19494,11 @@
       <c r="AK38" s="15" t="n"/>
       <c r="AL38" s="15" t="n"/>
       <c r="AM38" s="15" t="n"/>
-      <c r="AN38" s="15" t="n"/>
-      <c r="AO38" s="28" t="n"/>
-      <c r="AP38" s="15" t="n"/>
-      <c r="AQ38" s="15" t="n"/>
-      <c r="AR38" s="15" t="n"/>
+      <c r="AV38" s="15" t="n"/>
+      <c r="AW38" s="28" t="n"/>
+      <c r="AX38" s="15" t="n"/>
+      <c r="AY38" s="15" t="n"/>
+      <c r="AZ38" s="15" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="17" t="n"/>
@@ -19473,11 +19540,11 @@
       <c r="AK39" s="15" t="n"/>
       <c r="AL39" s="15" t="n"/>
       <c r="AM39" s="15" t="n"/>
-      <c r="AN39" s="15" t="n"/>
-      <c r="AO39" s="28" t="n"/>
-      <c r="AP39" s="15" t="n"/>
-      <c r="AQ39" s="15" t="n"/>
-      <c r="AR39" s="15" t="n"/>
+      <c r="AV39" s="15" t="n"/>
+      <c r="AW39" s="28" t="n"/>
+      <c r="AX39" s="15" t="n"/>
+      <c r="AY39" s="15" t="n"/>
+      <c r="AZ39" s="15" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="17" t="n"/>
@@ -19519,11 +19586,11 @@
       <c r="AK40" s="15" t="n"/>
       <c r="AL40" s="15" t="n"/>
       <c r="AM40" s="15" t="n"/>
-      <c r="AN40" s="15" t="n"/>
-      <c r="AO40" s="28" t="n"/>
-      <c r="AP40" s="15" t="n"/>
-      <c r="AQ40" s="15" t="n"/>
-      <c r="AR40" s="15" t="n"/>
+      <c r="AV40" s="15" t="n"/>
+      <c r="AW40" s="28" t="n"/>
+      <c r="AX40" s="15" t="n"/>
+      <c r="AY40" s="15" t="n"/>
+      <c r="AZ40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="17" t="n"/>
@@ -19565,11 +19632,11 @@
       <c r="AK41" s="15" t="n"/>
       <c r="AL41" s="15" t="n"/>
       <c r="AM41" s="15" t="n"/>
-      <c r="AN41" s="15" t="n"/>
-      <c r="AO41" s="28" t="n"/>
-      <c r="AP41" s="15" t="n"/>
-      <c r="AQ41" s="15" t="n"/>
-      <c r="AR41" s="15" t="n"/>
+      <c r="AV41" s="15" t="n"/>
+      <c r="AW41" s="28" t="n"/>
+      <c r="AX41" s="15" t="n"/>
+      <c r="AY41" s="15" t="n"/>
+      <c r="AZ41" s="15" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="17" t="n"/>
@@ -19611,11 +19678,11 @@
       <c r="AK42" s="15" t="n"/>
       <c r="AL42" s="15" t="n"/>
       <c r="AM42" s="15" t="n"/>
-      <c r="AN42" s="15" t="n"/>
-      <c r="AO42" s="28" t="n"/>
-      <c r="AP42" s="15" t="n"/>
-      <c r="AQ42" s="15" t="n"/>
-      <c r="AR42" s="15" t="n"/>
+      <c r="AV42" s="15" t="n"/>
+      <c r="AW42" s="28" t="n"/>
+      <c r="AX42" s="15" t="n"/>
+      <c r="AY42" s="15" t="n"/>
+      <c r="AZ42" s="15" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="n"/>
@@ -19657,11 +19724,11 @@
       <c r="AK43" s="15" t="n"/>
       <c r="AL43" s="15" t="n"/>
       <c r="AM43" s="15" t="n"/>
-      <c r="AN43" s="15" t="n"/>
-      <c r="AO43" s="28" t="n"/>
-      <c r="AP43" s="15" t="n"/>
-      <c r="AQ43" s="15" t="n"/>
-      <c r="AR43" s="15" t="n"/>
+      <c r="AV43" s="15" t="n"/>
+      <c r="AW43" s="28" t="n"/>
+      <c r="AX43" s="15" t="n"/>
+      <c r="AY43" s="15" t="n"/>
+      <c r="AZ43" s="15" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="17" t="n"/>
@@ -19703,11 +19770,11 @@
       <c r="AK44" s="15" t="n"/>
       <c r="AL44" s="15" t="n"/>
       <c r="AM44" s="15" t="n"/>
-      <c r="AN44" s="15" t="n"/>
-      <c r="AO44" s="28" t="n"/>
-      <c r="AP44" s="15" t="n"/>
-      <c r="AQ44" s="15" t="n"/>
-      <c r="AR44" s="15" t="n"/>
+      <c r="AV44" s="15" t="n"/>
+      <c r="AW44" s="28" t="n"/>
+      <c r="AX44" s="15" t="n"/>
+      <c r="AY44" s="15" t="n"/>
+      <c r="AZ44" s="15" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n"/>
@@ -19749,11 +19816,11 @@
       <c r="AK45" s="15" t="n"/>
       <c r="AL45" s="15" t="n"/>
       <c r="AM45" s="15" t="n"/>
-      <c r="AN45" s="15" t="n"/>
-      <c r="AO45" s="28" t="n"/>
-      <c r="AP45" s="15" t="n"/>
-      <c r="AQ45" s="15" t="n"/>
-      <c r="AR45" s="15" t="n"/>
+      <c r="AV45" s="15" t="n"/>
+      <c r="AW45" s="28" t="n"/>
+      <c r="AX45" s="15" t="n"/>
+      <c r="AY45" s="15" t="n"/>
+      <c r="AZ45" s="15" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="17" t="n"/>
@@ -19795,11 +19862,11 @@
       <c r="AK46" s="15" t="n"/>
       <c r="AL46" s="15" t="n"/>
       <c r="AM46" s="15" t="n"/>
-      <c r="AN46" s="15" t="n"/>
-      <c r="AO46" s="28" t="n"/>
-      <c r="AP46" s="15" t="n"/>
-      <c r="AQ46" s="15" t="n"/>
-      <c r="AR46" s="15" t="n"/>
+      <c r="AV46" s="15" t="n"/>
+      <c r="AW46" s="28" t="n"/>
+      <c r="AX46" s="15" t="n"/>
+      <c r="AY46" s="15" t="n"/>
+      <c r="AZ46" s="15" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="17" t="n"/>
@@ -19841,11 +19908,11 @@
       <c r="AK47" s="15" t="n"/>
       <c r="AL47" s="15" t="n"/>
       <c r="AM47" s="15" t="n"/>
-      <c r="AN47" s="15" t="n"/>
-      <c r="AO47" s="28" t="n"/>
-      <c r="AP47" s="15" t="n"/>
-      <c r="AQ47" s="15" t="n"/>
-      <c r="AR47" s="15" t="n"/>
+      <c r="AV47" s="15" t="n"/>
+      <c r="AW47" s="28" t="n"/>
+      <c r="AX47" s="15" t="n"/>
+      <c r="AY47" s="15" t="n"/>
+      <c r="AZ47" s="15" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="17" t="n"/>
@@ -19887,11 +19954,11 @@
       <c r="AK48" s="15" t="n"/>
       <c r="AL48" s="15" t="n"/>
       <c r="AM48" s="15" t="n"/>
-      <c r="AN48" s="15" t="n"/>
-      <c r="AO48" s="28" t="n"/>
-      <c r="AP48" s="15" t="n"/>
-      <c r="AQ48" s="15" t="n"/>
-      <c r="AR48" s="15" t="n"/>
+      <c r="AV48" s="15" t="n"/>
+      <c r="AW48" s="28" t="n"/>
+      <c r="AX48" s="15" t="n"/>
+      <c r="AY48" s="15" t="n"/>
+      <c r="AZ48" s="15" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n"/>
@@ -19933,11 +20000,11 @@
       <c r="AK49" s="15" t="n"/>
       <c r="AL49" s="15" t="n"/>
       <c r="AM49" s="15" t="n"/>
-      <c r="AN49" s="15" t="n"/>
-      <c r="AO49" s="28" t="n"/>
-      <c r="AP49" s="15" t="n"/>
-      <c r="AQ49" s="15" t="n"/>
-      <c r="AR49" s="15" t="n"/>
+      <c r="AV49" s="15" t="n"/>
+      <c r="AW49" s="28" t="n"/>
+      <c r="AX49" s="15" t="n"/>
+      <c r="AY49" s="15" t="n"/>
+      <c r="AZ49" s="15" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="17" t="n"/>
@@ -19979,11 +20046,11 @@
       <c r="AK50" s="15" t="n"/>
       <c r="AL50" s="15" t="n"/>
       <c r="AM50" s="15" t="n"/>
-      <c r="AN50" s="15" t="n"/>
-      <c r="AO50" s="28" t="n"/>
-      <c r="AP50" s="15" t="n"/>
-      <c r="AQ50" s="15" t="n"/>
-      <c r="AR50" s="15" t="n"/>
+      <c r="AV50" s="15" t="n"/>
+      <c r="AW50" s="28" t="n"/>
+      <c r="AX50" s="15" t="n"/>
+      <c r="AY50" s="15" t="n"/>
+      <c r="AZ50" s="15" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="17" t="n"/>
@@ -20025,11 +20092,11 @@
       <c r="AK51" s="15" t="n"/>
       <c r="AL51" s="15" t="n"/>
       <c r="AM51" s="15" t="n"/>
-      <c r="AN51" s="15" t="n"/>
-      <c r="AO51" s="28" t="n"/>
-      <c r="AP51" s="15" t="n"/>
-      <c r="AQ51" s="15" t="n"/>
-      <c r="AR51" s="15" t="n"/>
+      <c r="AV51" s="15" t="n"/>
+      <c r="AW51" s="28" t="n"/>
+      <c r="AX51" s="15" t="n"/>
+      <c r="AY51" s="15" t="n"/>
+      <c r="AZ51" s="15" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="17" t="n"/>
@@ -20071,11 +20138,11 @@
       <c r="AK52" s="15" t="n"/>
       <c r="AL52" s="15" t="n"/>
       <c r="AM52" s="15" t="n"/>
-      <c r="AN52" s="15" t="n"/>
-      <c r="AO52" s="28" t="n"/>
-      <c r="AP52" s="15" t="n"/>
-      <c r="AQ52" s="15" t="n"/>
-      <c r="AR52" s="15" t="n"/>
+      <c r="AV52" s="15" t="n"/>
+      <c r="AW52" s="28" t="n"/>
+      <c r="AX52" s="15" t="n"/>
+      <c r="AY52" s="15" t="n"/>
+      <c r="AZ52" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -20135,7 +20202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR52"/>
+  <dimension ref="A1:AZ55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="34.83203125" customWidth="1" style="2" min="1" max="1"/>
@@ -20352,13 +20419,13 @@
       <c r="AK15" s="20" t="n"/>
       <c r="AL15" s="20" t="n"/>
       <c r="AM15" s="21" t="n"/>
-      <c r="AP15" s="19" t="inlineStr">
+      <c r="AX15" s="19" t="inlineStr">
         <is>
           <t>Custom Properties</t>
         </is>
       </c>
-      <c r="AQ15" s="20" t="n"/>
-      <c r="AR15" s="20" t="n"/>
+      <c r="AY15" s="20" t="n"/>
+      <c r="AZ15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -20556,19 +20623,59 @@
           <t>Pattern</t>
         </is>
       </c>
-      <c r="AN16" s="10" t="inlineStr">
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>Element Type</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Distance Metric</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Normalized</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>Embedding Model</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>Embedding Model Version</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Default Timezone</t>
+        </is>
+      </c>
+      <c r="AV16" s="10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="AO16" s="10" t="inlineStr">
+      <c r="AW16" s="10" t="inlineStr">
         <is>
           <t>Comments (internal)</t>
         </is>
       </c>
-      <c r="AP16" s="10" t="n"/>
-      <c r="AQ16" s="10" t="n"/>
-      <c r="AR16" s="10" t="n"/>
+      <c r="AX16" s="10" t="n"/>
+      <c r="AY16" s="10" t="n"/>
+      <c r="AZ16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -20676,15 +20783,15 @@
       <c r="AK17" s="15" t="n"/>
       <c r="AL17" s="15" t="n"/>
       <c r="AM17" s="15" t="n"/>
-      <c r="AN17" s="15" t="inlineStr">
+      <c r="AV17" s="15" t="inlineStr">
         <is>
           <t>shipmentsShipmentId</t>
         </is>
       </c>
-      <c r="AO17" s="28" t="n"/>
-      <c r="AP17" s="15" t="n"/>
-      <c r="AQ17" s="15" t="n"/>
-      <c r="AR17" s="15" t="n"/>
+      <c r="AW17" s="28" t="n"/>
+      <c r="AX17" s="15" t="n"/>
+      <c r="AY17" s="15" t="n"/>
+      <c r="AZ17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -20768,15 +20875,15 @@
           <t>^ORD[0-9]+$</t>
         </is>
       </c>
-      <c r="AN18" s="15" t="inlineStr">
+      <c r="AV18" s="15" t="inlineStr">
         <is>
           <t>shipmentsOrderId</t>
         </is>
       </c>
-      <c r="AO18" s="28" t="n"/>
-      <c r="AP18" s="15" t="n"/>
-      <c r="AQ18" s="15" t="n"/>
-      <c r="AR18" s="15" t="n"/>
+      <c r="AW18" s="28" t="n"/>
+      <c r="AX18" s="15" t="n"/>
+      <c r="AY18" s="15" t="n"/>
+      <c r="AZ18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -20854,15 +20961,15 @@
       <c r="AK19" s="15" t="n"/>
       <c r="AL19" s="15" t="n"/>
       <c r="AM19" s="15" t="n"/>
-      <c r="AN19" s="15" t="inlineStr">
+      <c r="AV19" s="15" t="inlineStr">
         <is>
           <t>shipmentsShippedDate</t>
         </is>
       </c>
-      <c r="AO19" s="28" t="n"/>
-      <c r="AP19" s="15" t="n"/>
-      <c r="AQ19" s="15" t="n"/>
-      <c r="AR19" s="15" t="n"/>
+      <c r="AW19" s="28" t="n"/>
+      <c r="AX19" s="15" t="n"/>
+      <c r="AY19" s="15" t="n"/>
+      <c r="AZ19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
@@ -20936,15 +21043,23 @@
       <c r="AK20" s="15" t="n"/>
       <c r="AL20" s="15" t="n"/>
       <c r="AM20" s="15" t="n"/>
-      <c r="AN20" s="15" t="inlineStr">
+      <c r="AT20" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="AV20" s="15" t="inlineStr">
         <is>
           <t>shipmentsDeliveredTs</t>
         </is>
       </c>
-      <c r="AO20" s="28" t="n"/>
-      <c r="AP20" s="15" t="n"/>
-      <c r="AQ20" s="15" t="n"/>
-      <c r="AR20" s="15" t="n"/>
+      <c r="AW20" s="28" t="n"/>
+      <c r="AX20" s="15" t="n"/>
+      <c r="AY20" s="15" t="n"/>
+      <c r="AZ20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
@@ -21030,15 +21145,15 @@
       <c r="AK21" s="15" t="n"/>
       <c r="AL21" s="15" t="n"/>
       <c r="AM21" s="15" t="n"/>
-      <c r="AN21" s="15" t="inlineStr">
+      <c r="AV21" s="15" t="inlineStr">
         <is>
           <t>shipmentsCarrier</t>
         </is>
       </c>
-      <c r="AO21" s="28" t="n"/>
-      <c r="AP21" s="15" t="n"/>
-      <c r="AQ21" s="15" t="n"/>
-      <c r="AR21" s="15" t="n"/>
+      <c r="AW21" s="28" t="n"/>
+      <c r="AX21" s="15" t="n"/>
+      <c r="AY21" s="15" t="n"/>
+      <c r="AZ21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
@@ -21112,15 +21227,15 @@
       <c r="AK22" s="15" t="n"/>
       <c r="AL22" s="15" t="n"/>
       <c r="AM22" s="15" t="n"/>
-      <c r="AN22" s="15" t="inlineStr">
+      <c r="AV22" s="15" t="inlineStr">
         <is>
           <t>shipmentsStatus</t>
         </is>
       </c>
-      <c r="AO22" s="28" t="n"/>
-      <c r="AP22" s="15" t="n"/>
-      <c r="AQ22" s="15" t="n"/>
-      <c r="AR22" s="15" t="n"/>
+      <c r="AW22" s="28" t="n"/>
+      <c r="AX22" s="15" t="n"/>
+      <c r="AY22" s="15" t="n"/>
+      <c r="AZ22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
@@ -21194,15 +21309,15 @@
       <c r="AK23" s="15" t="n"/>
       <c r="AL23" s="15" t="n"/>
       <c r="AM23" s="15" t="n"/>
-      <c r="AN23" s="15" t="inlineStr">
+      <c r="AV23" s="15" t="inlineStr">
         <is>
           <t>shipmentsParcelCount</t>
         </is>
       </c>
-      <c r="AO23" s="28" t="n"/>
-      <c r="AP23" s="15" t="n"/>
-      <c r="AQ23" s="15" t="n"/>
-      <c r="AR23" s="15" t="n"/>
+      <c r="AW23" s="28" t="n"/>
+      <c r="AX23" s="15" t="n"/>
+      <c r="AY23" s="15" t="n"/>
+      <c r="AZ23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -21292,15 +21407,15 @@
       <c r="AK24" s="15" t="n"/>
       <c r="AL24" s="15" t="n"/>
       <c r="AM24" s="15" t="n"/>
-      <c r="AN24" s="15" t="inlineStr">
+      <c r="AV24" s="15" t="inlineStr">
         <is>
           <t>shipmentsShippingCost</t>
         </is>
       </c>
-      <c r="AO24" s="28" t="n"/>
-      <c r="AP24" s="15" t="n"/>
-      <c r="AQ24" s="15" t="n"/>
-      <c r="AR24" s="15" t="n"/>
+      <c r="AW24" s="28" t="n"/>
+      <c r="AX24" s="15" t="n"/>
+      <c r="AY24" s="15" t="n"/>
+      <c r="AZ24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
@@ -21368,15 +21483,15 @@
       <c r="AK25" s="15" t="n"/>
       <c r="AL25" s="15" t="n"/>
       <c r="AM25" s="15" t="n"/>
-      <c r="AN25" s="15" t="inlineStr">
+      <c r="AV25" s="15" t="inlineStr">
         <is>
           <t>shipmentsIsExpress</t>
         </is>
       </c>
-      <c r="AO25" s="28" t="n"/>
-      <c r="AP25" s="15" t="n"/>
-      <c r="AQ25" s="15" t="n"/>
-      <c r="AR25" s="15" t="n"/>
+      <c r="AW25" s="28" t="n"/>
+      <c r="AX25" s="15" t="n"/>
+      <c r="AY25" s="15" t="n"/>
+      <c r="AZ25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
@@ -21448,15 +21563,15 @@
       <c r="AK26" s="15" t="n"/>
       <c r="AL26" s="15" t="n"/>
       <c r="AM26" s="15" t="n"/>
-      <c r="AN26" s="15" t="inlineStr">
+      <c r="AV26" s="15" t="inlineStr">
         <is>
           <t>shipmentsLegacyStatus</t>
         </is>
       </c>
-      <c r="AO26" s="28" t="n"/>
-      <c r="AP26" s="15" t="n"/>
-      <c r="AQ26" s="15" t="n"/>
-      <c r="AR26" s="15" t="n"/>
+      <c r="AW26" s="28" t="n"/>
+      <c r="AX26" s="15" t="n"/>
+      <c r="AY26" s="15" t="n"/>
+      <c r="AZ26" s="15" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
@@ -21532,15 +21647,15 @@
         </is>
       </c>
       <c r="AM27" s="15" t="n"/>
-      <c r="AN27" s="15" t="inlineStr">
+      <c r="AV27" s="15" t="inlineStr">
         <is>
           <t>shipmentsAddress</t>
         </is>
       </c>
-      <c r="AO27" s="28" t="n"/>
-      <c r="AP27" s="15" t="n"/>
-      <c r="AQ27" s="15" t="n"/>
-      <c r="AR27" s="15" t="n"/>
+      <c r="AW27" s="28" t="n"/>
+      <c r="AX27" s="15" t="n"/>
+      <c r="AY27" s="15" t="n"/>
+      <c r="AZ27" s="15" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
@@ -21608,15 +21723,15 @@
       <c r="AK28" s="15" t="n"/>
       <c r="AL28" s="15" t="n"/>
       <c r="AM28" s="15" t="n"/>
-      <c r="AN28" s="15" t="inlineStr">
+      <c r="AV28" s="15" t="inlineStr">
         <is>
           <t>addressStreet</t>
         </is>
       </c>
-      <c r="AO28" s="28" t="n"/>
-      <c r="AP28" s="15" t="n"/>
-      <c r="AQ28" s="15" t="n"/>
-      <c r="AR28" s="15" t="n"/>
+      <c r="AW28" s="28" t="n"/>
+      <c r="AX28" s="15" t="n"/>
+      <c r="AY28" s="15" t="n"/>
+      <c r="AZ28" s="15" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
@@ -21684,15 +21799,15 @@
       <c r="AK29" s="15" t="n"/>
       <c r="AL29" s="15" t="n"/>
       <c r="AM29" s="15" t="n"/>
-      <c r="AN29" s="15" t="inlineStr">
+      <c r="AV29" s="15" t="inlineStr">
         <is>
           <t>addressCity</t>
         </is>
       </c>
-      <c r="AO29" s="28" t="n"/>
-      <c r="AP29" s="15" t="n"/>
-      <c r="AQ29" s="15" t="n"/>
-      <c r="AR29" s="15" t="n"/>
+      <c r="AW29" s="28" t="n"/>
+      <c r="AX29" s="15" t="n"/>
+      <c r="AY29" s="15" t="n"/>
+      <c r="AZ29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -21762,15 +21877,15 @@
       <c r="AK30" s="15" t="n"/>
       <c r="AL30" s="15" t="n"/>
       <c r="AM30" s="15" t="n"/>
-      <c r="AN30" s="15" t="inlineStr">
+      <c r="AV30" s="15" t="inlineStr">
         <is>
           <t>addressCountry</t>
         </is>
       </c>
-      <c r="AO30" s="28" t="n"/>
-      <c r="AP30" s="15" t="n"/>
-      <c r="AQ30" s="15" t="n"/>
-      <c r="AR30" s="15" t="n"/>
+      <c r="AW30" s="28" t="n"/>
+      <c r="AX30" s="15" t="n"/>
+      <c r="AY30" s="15" t="n"/>
+      <c r="AZ30" s="15" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -21828,15 +21943,15 @@
       <c r="AK31" s="15" t="n"/>
       <c r="AL31" s="15" t="n"/>
       <c r="AM31" s="15" t="n"/>
-      <c r="AN31" s="15" t="inlineStr">
+      <c r="AV31" s="15" t="inlineStr">
         <is>
           <t>addressGeo</t>
         </is>
       </c>
-      <c r="AO31" s="28" t="n"/>
-      <c r="AP31" s="15" t="n"/>
-      <c r="AQ31" s="15" t="n"/>
-      <c r="AR31" s="15" t="n"/>
+      <c r="AW31" s="28" t="n"/>
+      <c r="AX31" s="15" t="n"/>
+      <c r="AY31" s="15" t="n"/>
+      <c r="AZ31" s="15" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
@@ -21892,15 +22007,15 @@
       <c r="AK32" s="15" t="n"/>
       <c r="AL32" s="15" t="n"/>
       <c r="AM32" s="15" t="n"/>
-      <c r="AN32" s="15" t="inlineStr">
+      <c r="AV32" s="15" t="inlineStr">
         <is>
           <t>geoLatitude</t>
         </is>
       </c>
-      <c r="AO32" s="28" t="n"/>
-      <c r="AP32" s="15" t="n"/>
-      <c r="AQ32" s="15" t="n"/>
-      <c r="AR32" s="15" t="n"/>
+      <c r="AW32" s="28" t="n"/>
+      <c r="AX32" s="15" t="n"/>
+      <c r="AY32" s="15" t="n"/>
+      <c r="AZ32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
@@ -21956,15 +22071,15 @@
       <c r="AK33" s="15" t="n"/>
       <c r="AL33" s="15" t="n"/>
       <c r="AM33" s="15" t="n"/>
-      <c r="AN33" s="15" t="inlineStr">
+      <c r="AV33" s="15" t="inlineStr">
         <is>
           <t>geoLongitude</t>
         </is>
       </c>
-      <c r="AO33" s="28" t="n"/>
-      <c r="AP33" s="15" t="n"/>
-      <c r="AQ33" s="15" t="n"/>
-      <c r="AR33" s="15" t="n"/>
+      <c r="AW33" s="28" t="n"/>
+      <c r="AX33" s="15" t="n"/>
+      <c r="AY33" s="15" t="n"/>
+      <c r="AZ33" s="15" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
@@ -22036,115 +22151,61 @@
       <c r="AK34" s="15" t="n"/>
       <c r="AL34" s="15" t="n"/>
       <c r="AM34" s="15" t="n"/>
-      <c r="AN34" s="15" t="inlineStr">
+      <c r="AV34" s="15" t="inlineStr">
         <is>
           <t>shipmentsHandlingTags</t>
         </is>
       </c>
-      <c r="AO34" s="28" t="n"/>
-      <c r="AP34" s="15" t="n"/>
-      <c r="AQ34" s="15" t="n"/>
-      <c r="AR34" s="15" t="n"/>
+      <c r="AW34" s="28" t="n"/>
+      <c r="AX34" s="15" t="n"/>
+      <c r="AY34" s="15" t="n"/>
+      <c r="AZ34" s="15" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>attributes</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="inlineStr">
-        <is>
-          <t>Attributes</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="15" t="inlineStr">
-        <is>
-          <t>Free-form key/value attributes.</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="n"/>
-      <c r="H35" s="15" t="n"/>
-      <c r="I35" s="15" t="inlineStr">
-        <is>
-          <t>internal</t>
-        </is>
-      </c>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15" t="n"/>
-      <c r="L35" s="15" t="n"/>
-      <c r="M35" s="15" t="n"/>
-      <c r="N35" s="15" t="n"/>
-      <c r="O35" s="15" t="n"/>
-      <c r="P35" s="15" t="n"/>
-      <c r="Q35" s="15" t="n"/>
-      <c r="R35" s="15" t="n"/>
-      <c r="S35" s="15" t="n"/>
-      <c r="T35" s="15" t="n"/>
-      <c r="U35" s="15" t="n"/>
-      <c r="V35" s="15" t="n"/>
-      <c r="W35" s="15" t="n"/>
-      <c r="X35" s="15" t="n"/>
-      <c r="Y35" s="15" t="n"/>
-      <c r="Z35" s="15" t="n"/>
-      <c r="AA35" s="15" t="n"/>
-      <c r="AB35" s="15" t="n"/>
-      <c r="AC35" s="15" t="n"/>
-      <c r="AD35" s="15" t="n"/>
-      <c r="AE35" s="15" t="n"/>
-      <c r="AF35" s="15" t="n"/>
-      <c r="AG35" s="15" t="n"/>
-      <c r="AH35" s="15" t="n"/>
-      <c r="AI35" s="15" t="n"/>
-      <c r="AJ35" s="15" t="n"/>
-      <c r="AK35" s="15" t="n"/>
-      <c r="AL35" s="15" t="n"/>
-      <c r="AM35" s="15" t="n"/>
-      <c r="AN35" s="15" t="inlineStr">
-        <is>
-          <t>shipmentsAttributes</t>
-        </is>
-      </c>
-      <c r="AO35" s="28" t="n"/>
-      <c r="AP35" s="15" t="n"/>
-      <c r="AQ35" s="15" t="n"/>
-      <c r="AR35" s="15" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>handling_tags.items</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="AD35" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>description_embedding</t>
+          <t>attributes</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>Description Embedding</t>
+          <t>Attributes</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>map</t>
         </is>
       </c>
       <c r="E36" s="16" t="n"/>
       <c r="F36" s="15" t="inlineStr">
         <is>
-          <t>Embedding of the shipment description.</t>
+          <t>Free-form key/value attributes.</t>
         </is>
       </c>
       <c r="G36" s="15" t="n"/>
@@ -22184,146 +22245,84 @@
       <c r="AK36" s="15" t="n"/>
       <c r="AL36" s="15" t="n"/>
       <c r="AM36" s="15" t="n"/>
-      <c r="AN36" s="15" t="inlineStr">
-        <is>
-          <t>shipmentsEmbedding</t>
-        </is>
-      </c>
-      <c r="AO36" s="28" t="n"/>
-      <c r="AP36" s="15" t="n"/>
-      <c r="AQ36" s="15" t="n"/>
-      <c r="AR36" s="15" t="n"/>
+      <c r="AV36" s="15" t="inlineStr">
+        <is>
+          <t>shipmentsAttributes</t>
+        </is>
+      </c>
+      <c r="AW36" s="28" t="n"/>
+      <c r="AX36" s="15" t="n"/>
+      <c r="AY36" s="15" t="n"/>
+      <c r="AZ36" s="15" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>delivery_note</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>Delivery Note</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>attributes.key</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="15" t="inlineStr">
-        <is>
-          <t>Free-text note captured at handover.</t>
-        </is>
-      </c>
-      <c r="G37" s="15" t="n"/>
-      <c r="H37" s="15" t="n"/>
-      <c r="I37" s="15" t="inlineStr">
-        <is>
-          <t>restricted</t>
-        </is>
-      </c>
-      <c r="J37" s="15" t="n"/>
-      <c r="K37" s="15" t="n"/>
-      <c r="L37" s="15" t="n"/>
-      <c r="M37" s="15" t="n"/>
-      <c r="N37" s="15" t="n"/>
-      <c r="O37" s="15" t="n"/>
-      <c r="P37" s="15" t="n"/>
-      <c r="Q37" s="15" t="n"/>
-      <c r="R37" s="15" t="n"/>
-      <c r="S37" s="15" t="n"/>
-      <c r="T37" s="15" t="n"/>
-      <c r="U37" s="15" t="n"/>
-      <c r="V37" s="15" t="n"/>
-      <c r="W37" s="15" t="n"/>
-      <c r="X37" s="15" t="n"/>
-      <c r="Y37" s="15" t="n"/>
-      <c r="Z37" s="15" t="n"/>
-      <c r="AA37" s="15" t="n"/>
-      <c r="AB37" s="15" t="n"/>
-      <c r="AC37" s="15" t="n"/>
-      <c r="AD37" s="15" t="n"/>
-      <c r="AE37" s="15" t="n"/>
-      <c r="AF37" s="15" t="n"/>
-      <c r="AG37" s="15" t="n"/>
-      <c r="AH37" s="15" t="n"/>
-      <c r="AI37" s="15" t="n"/>
-      <c r="AJ37" s="15" t="n"/>
-      <c r="AK37" s="15" t="n"/>
-      <c r="AL37" s="15" t="n"/>
-      <c r="AM37" s="15" t="n"/>
-      <c r="AN37" s="15" t="inlineStr">
-        <is>
-          <t>shipmentsDeliveryNote</t>
-        </is>
-      </c>
-      <c r="AO37" s="28" t="n"/>
-      <c r="AP37" s="15" t="n"/>
-      <c r="AQ37" s="15" t="n"/>
-      <c r="AR37" s="15" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="n"/>
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="15" t="n"/>
-      <c r="I38" s="15" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="15" t="n"/>
-      <c r="L38" s="15" t="n"/>
-      <c r="M38" s="15" t="n"/>
-      <c r="N38" s="15" t="n"/>
-      <c r="O38" s="15" t="n"/>
-      <c r="P38" s="15" t="n"/>
-      <c r="Q38" s="15" t="n"/>
-      <c r="R38" s="15" t="n"/>
-      <c r="S38" s="15" t="n"/>
-      <c r="T38" s="15" t="n"/>
-      <c r="U38" s="15" t="n"/>
-      <c r="V38" s="15" t="n"/>
-      <c r="W38" s="15" t="n"/>
-      <c r="X38" s="15" t="n"/>
-      <c r="Y38" s="15" t="n"/>
-      <c r="Z38" s="15" t="n"/>
-      <c r="AA38" s="15" t="n"/>
-      <c r="AB38" s="15" t="n"/>
-      <c r="AC38" s="15" t="n"/>
-      <c r="AD38" s="15" t="n"/>
-      <c r="AE38" s="15" t="n"/>
-      <c r="AF38" s="15" t="n"/>
-      <c r="AG38" s="15" t="n"/>
-      <c r="AH38" s="15" t="n"/>
-      <c r="AI38" s="15" t="n"/>
-      <c r="AJ38" s="15" t="n"/>
-      <c r="AK38" s="15" t="n"/>
-      <c r="AL38" s="15" t="n"/>
-      <c r="AM38" s="15" t="n"/>
-      <c r="AN38" s="15" t="n"/>
-      <c r="AO38" s="28" t="n"/>
-      <c r="AP38" s="15" t="n"/>
-      <c r="AQ38" s="15" t="n"/>
-      <c r="AR38" s="15" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>attributes.value</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="n"/>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>description_embedding</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Description Embedding</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
       <c r="E39" s="16" t="n"/>
-      <c r="F39" s="15" t="n"/>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>Embedding of the shipment description.</t>
+        </is>
+      </c>
       <c r="G39" s="15" t="n"/>
       <c r="H39" s="15" t="n"/>
-      <c r="I39" s="15" t="n"/>
+      <c r="I39" s="15" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
       <c r="J39" s="15" t="n"/>
       <c r="K39" s="15" t="n"/>
       <c r="L39" s="15" t="n"/>
@@ -22354,22 +22353,76 @@
       <c r="AK39" s="15" t="n"/>
       <c r="AL39" s="15" t="n"/>
       <c r="AM39" s="15" t="n"/>
-      <c r="AN39" s="15" t="n"/>
-      <c r="AO39" s="28" t="n"/>
-      <c r="AP39" s="15" t="n"/>
-      <c r="AQ39" s="15" t="n"/>
-      <c r="AR39" s="15" t="n"/>
+      <c r="AN39" t="n">
+        <v>1536</v>
+      </c>
+      <c r="AO39" t="inlineStr">
+        <is>
+          <t>float32</t>
+        </is>
+      </c>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>cosine</t>
+        </is>
+      </c>
+      <c r="AQ39" t="b">
+        <v>1</v>
+      </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>text-embedding-3-small</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AV39" s="15" t="inlineStr">
+        <is>
+          <t>shipmentsEmbedding</t>
+        </is>
+      </c>
+      <c r="AW39" s="28" t="n"/>
+      <c r="AX39" s="15" t="n"/>
+      <c r="AY39" s="15" t="n"/>
+      <c r="AZ39" s="15" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="n"/>
-      <c r="B40" s="15" t="n"/>
-      <c r="C40" s="15" t="n"/>
-      <c r="D40" s="15" t="n"/>
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>delivery_note</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>Delivery Note</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
       <c r="E40" s="16" t="n"/>
-      <c r="F40" s="15" t="n"/>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>Free-text note captured at handover.</t>
+        </is>
+      </c>
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="15" t="n"/>
-      <c r="I40" s="15" t="n"/>
+      <c r="I40" s="15" t="inlineStr">
+        <is>
+          <t>restricted</t>
+        </is>
+      </c>
       <c r="J40" s="15" t="n"/>
       <c r="K40" s="15" t="n"/>
       <c r="L40" s="15" t="n"/>
@@ -22400,11 +22453,15 @@
       <c r="AK40" s="15" t="n"/>
       <c r="AL40" s="15" t="n"/>
       <c r="AM40" s="15" t="n"/>
-      <c r="AN40" s="15" t="n"/>
-      <c r="AO40" s="28" t="n"/>
-      <c r="AP40" s="15" t="n"/>
-      <c r="AQ40" s="15" t="n"/>
-      <c r="AR40" s="15" t="n"/>
+      <c r="AV40" s="15" t="inlineStr">
+        <is>
+          <t>shipmentsDeliveryNote</t>
+        </is>
+      </c>
+      <c r="AW40" s="28" t="n"/>
+      <c r="AX40" s="15" t="n"/>
+      <c r="AY40" s="15" t="n"/>
+      <c r="AZ40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="17" t="n"/>
@@ -22446,11 +22503,11 @@
       <c r="AK41" s="15" t="n"/>
       <c r="AL41" s="15" t="n"/>
       <c r="AM41" s="15" t="n"/>
-      <c r="AN41" s="15" t="n"/>
-      <c r="AO41" s="28" t="n"/>
-      <c r="AP41" s="15" t="n"/>
-      <c r="AQ41" s="15" t="n"/>
-      <c r="AR41" s="15" t="n"/>
+      <c r="AV41" s="15" t="n"/>
+      <c r="AW41" s="28" t="n"/>
+      <c r="AX41" s="15" t="n"/>
+      <c r="AY41" s="15" t="n"/>
+      <c r="AZ41" s="15" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="17" t="n"/>
@@ -22492,11 +22549,11 @@
       <c r="AK42" s="15" t="n"/>
       <c r="AL42" s="15" t="n"/>
       <c r="AM42" s="15" t="n"/>
-      <c r="AN42" s="15" t="n"/>
-      <c r="AO42" s="28" t="n"/>
-      <c r="AP42" s="15" t="n"/>
-      <c r="AQ42" s="15" t="n"/>
-      <c r="AR42" s="15" t="n"/>
+      <c r="AV42" s="15" t="n"/>
+      <c r="AW42" s="28" t="n"/>
+      <c r="AX42" s="15" t="n"/>
+      <c r="AY42" s="15" t="n"/>
+      <c r="AZ42" s="15" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="n"/>
@@ -22538,11 +22595,11 @@
       <c r="AK43" s="15" t="n"/>
       <c r="AL43" s="15" t="n"/>
       <c r="AM43" s="15" t="n"/>
-      <c r="AN43" s="15" t="n"/>
-      <c r="AO43" s="28" t="n"/>
-      <c r="AP43" s="15" t="n"/>
-      <c r="AQ43" s="15" t="n"/>
-      <c r="AR43" s="15" t="n"/>
+      <c r="AV43" s="15" t="n"/>
+      <c r="AW43" s="28" t="n"/>
+      <c r="AX43" s="15" t="n"/>
+      <c r="AY43" s="15" t="n"/>
+      <c r="AZ43" s="15" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="17" t="n"/>
@@ -22584,11 +22641,11 @@
       <c r="AK44" s="15" t="n"/>
       <c r="AL44" s="15" t="n"/>
       <c r="AM44" s="15" t="n"/>
-      <c r="AN44" s="15" t="n"/>
-      <c r="AO44" s="28" t="n"/>
-      <c r="AP44" s="15" t="n"/>
-      <c r="AQ44" s="15" t="n"/>
-      <c r="AR44" s="15" t="n"/>
+      <c r="AV44" s="15" t="n"/>
+      <c r="AW44" s="28" t="n"/>
+      <c r="AX44" s="15" t="n"/>
+      <c r="AY44" s="15" t="n"/>
+      <c r="AZ44" s="15" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n"/>
@@ -22630,11 +22687,11 @@
       <c r="AK45" s="15" t="n"/>
       <c r="AL45" s="15" t="n"/>
       <c r="AM45" s="15" t="n"/>
-      <c r="AN45" s="15" t="n"/>
-      <c r="AO45" s="28" t="n"/>
-      <c r="AP45" s="15" t="n"/>
-      <c r="AQ45" s="15" t="n"/>
-      <c r="AR45" s="15" t="n"/>
+      <c r="AV45" s="15" t="n"/>
+      <c r="AW45" s="28" t="n"/>
+      <c r="AX45" s="15" t="n"/>
+      <c r="AY45" s="15" t="n"/>
+      <c r="AZ45" s="15" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="17" t="n"/>
@@ -22676,11 +22733,11 @@
       <c r="AK46" s="15" t="n"/>
       <c r="AL46" s="15" t="n"/>
       <c r="AM46" s="15" t="n"/>
-      <c r="AN46" s="15" t="n"/>
-      <c r="AO46" s="28" t="n"/>
-      <c r="AP46" s="15" t="n"/>
-      <c r="AQ46" s="15" t="n"/>
-      <c r="AR46" s="15" t="n"/>
+      <c r="AV46" s="15" t="n"/>
+      <c r="AW46" s="28" t="n"/>
+      <c r="AX46" s="15" t="n"/>
+      <c r="AY46" s="15" t="n"/>
+      <c r="AZ46" s="15" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="17" t="n"/>
@@ -22722,11 +22779,11 @@
       <c r="AK47" s="15" t="n"/>
       <c r="AL47" s="15" t="n"/>
       <c r="AM47" s="15" t="n"/>
-      <c r="AN47" s="15" t="n"/>
-      <c r="AO47" s="28" t="n"/>
-      <c r="AP47" s="15" t="n"/>
-      <c r="AQ47" s="15" t="n"/>
-      <c r="AR47" s="15" t="n"/>
+      <c r="AV47" s="15" t="n"/>
+      <c r="AW47" s="28" t="n"/>
+      <c r="AX47" s="15" t="n"/>
+      <c r="AY47" s="15" t="n"/>
+      <c r="AZ47" s="15" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="17" t="n"/>
@@ -22768,11 +22825,11 @@
       <c r="AK48" s="15" t="n"/>
       <c r="AL48" s="15" t="n"/>
       <c r="AM48" s="15" t="n"/>
-      <c r="AN48" s="15" t="n"/>
-      <c r="AO48" s="28" t="n"/>
-      <c r="AP48" s="15" t="n"/>
-      <c r="AQ48" s="15" t="n"/>
-      <c r="AR48" s="15" t="n"/>
+      <c r="AV48" s="15" t="n"/>
+      <c r="AW48" s="28" t="n"/>
+      <c r="AX48" s="15" t="n"/>
+      <c r="AY48" s="15" t="n"/>
+      <c r="AZ48" s="15" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n"/>
@@ -22814,11 +22871,11 @@
       <c r="AK49" s="15" t="n"/>
       <c r="AL49" s="15" t="n"/>
       <c r="AM49" s="15" t="n"/>
-      <c r="AN49" s="15" t="n"/>
-      <c r="AO49" s="28" t="n"/>
-      <c r="AP49" s="15" t="n"/>
-      <c r="AQ49" s="15" t="n"/>
-      <c r="AR49" s="15" t="n"/>
+      <c r="AV49" s="15" t="n"/>
+      <c r="AW49" s="28" t="n"/>
+      <c r="AX49" s="15" t="n"/>
+      <c r="AY49" s="15" t="n"/>
+      <c r="AZ49" s="15" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="17" t="n"/>
@@ -22860,11 +22917,11 @@
       <c r="AK50" s="15" t="n"/>
       <c r="AL50" s="15" t="n"/>
       <c r="AM50" s="15" t="n"/>
-      <c r="AN50" s="15" t="n"/>
-      <c r="AO50" s="28" t="n"/>
-      <c r="AP50" s="15" t="n"/>
-      <c r="AQ50" s="15" t="n"/>
-      <c r="AR50" s="15" t="n"/>
+      <c r="AV50" s="15" t="n"/>
+      <c r="AW50" s="28" t="n"/>
+      <c r="AX50" s="15" t="n"/>
+      <c r="AY50" s="15" t="n"/>
+      <c r="AZ50" s="15" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="17" t="n"/>
@@ -22906,11 +22963,11 @@
       <c r="AK51" s="15" t="n"/>
       <c r="AL51" s="15" t="n"/>
       <c r="AM51" s="15" t="n"/>
-      <c r="AN51" s="15" t="n"/>
-      <c r="AO51" s="28" t="n"/>
-      <c r="AP51" s="15" t="n"/>
-      <c r="AQ51" s="15" t="n"/>
-      <c r="AR51" s="15" t="n"/>
+      <c r="AV51" s="15" t="n"/>
+      <c r="AW51" s="28" t="n"/>
+      <c r="AX51" s="15" t="n"/>
+      <c r="AY51" s="15" t="n"/>
+      <c r="AZ51" s="15" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="17" t="n"/>
@@ -22952,11 +23009,149 @@
       <c r="AK52" s="15" t="n"/>
       <c r="AL52" s="15" t="n"/>
       <c r="AM52" s="15" t="n"/>
-      <c r="AN52" s="15" t="n"/>
-      <c r="AO52" s="28" t="n"/>
-      <c r="AP52" s="15" t="n"/>
-      <c r="AQ52" s="15" t="n"/>
-      <c r="AR52" s="15" t="n"/>
+      <c r="AV52" s="15" t="n"/>
+      <c r="AW52" s="28" t="n"/>
+      <c r="AX52" s="15" t="n"/>
+      <c r="AY52" s="15" t="n"/>
+      <c r="AZ52" s="15" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n"/>
+      <c r="B53" s="15" t="n"/>
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="16" t="n"/>
+      <c r="F53" s="15" t="n"/>
+      <c r="G53" s="15" t="n"/>
+      <c r="H53" s="15" t="n"/>
+      <c r="I53" s="15" t="n"/>
+      <c r="J53" s="15" t="n"/>
+      <c r="K53" s="15" t="n"/>
+      <c r="L53" s="15" t="n"/>
+      <c r="M53" s="15" t="n"/>
+      <c r="N53" s="15" t="n"/>
+      <c r="O53" s="15" t="n"/>
+      <c r="P53" s="15" t="n"/>
+      <c r="Q53" s="15" t="n"/>
+      <c r="R53" s="15" t="n"/>
+      <c r="S53" s="15" t="n"/>
+      <c r="T53" s="15" t="n"/>
+      <c r="U53" s="15" t="n"/>
+      <c r="V53" s="15" t="n"/>
+      <c r="W53" s="15" t="n"/>
+      <c r="X53" s="15" t="n"/>
+      <c r="Y53" s="15" t="n"/>
+      <c r="Z53" s="15" t="n"/>
+      <c r="AA53" s="15" t="n"/>
+      <c r="AB53" s="15" t="n"/>
+      <c r="AC53" s="15" t="n"/>
+      <c r="AD53" s="15" t="n"/>
+      <c r="AE53" s="15" t="n"/>
+      <c r="AF53" s="15" t="n"/>
+      <c r="AG53" s="15" t="n"/>
+      <c r="AH53" s="15" t="n"/>
+      <c r="AI53" s="15" t="n"/>
+      <c r="AJ53" s="15" t="n"/>
+      <c r="AK53" s="15" t="n"/>
+      <c r="AL53" s="15" t="n"/>
+      <c r="AM53" s="15" t="n"/>
+      <c r="AV53" s="15" t="n"/>
+      <c r="AW53" s="28" t="n"/>
+      <c r="AX53" s="15" t="n"/>
+      <c r="AY53" s="15" t="n"/>
+      <c r="AZ53" s="15" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="n"/>
+      <c r="B54" s="15" t="n"/>
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="16" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="15" t="n"/>
+      <c r="H54" s="15" t="n"/>
+      <c r="I54" s="15" t="n"/>
+      <c r="J54" s="15" t="n"/>
+      <c r="K54" s="15" t="n"/>
+      <c r="L54" s="15" t="n"/>
+      <c r="M54" s="15" t="n"/>
+      <c r="N54" s="15" t="n"/>
+      <c r="O54" s="15" t="n"/>
+      <c r="P54" s="15" t="n"/>
+      <c r="Q54" s="15" t="n"/>
+      <c r="R54" s="15" t="n"/>
+      <c r="S54" s="15" t="n"/>
+      <c r="T54" s="15" t="n"/>
+      <c r="U54" s="15" t="n"/>
+      <c r="V54" s="15" t="n"/>
+      <c r="W54" s="15" t="n"/>
+      <c r="X54" s="15" t="n"/>
+      <c r="Y54" s="15" t="n"/>
+      <c r="Z54" s="15" t="n"/>
+      <c r="AA54" s="15" t="n"/>
+      <c r="AB54" s="15" t="n"/>
+      <c r="AC54" s="15" t="n"/>
+      <c r="AD54" s="15" t="n"/>
+      <c r="AE54" s="15" t="n"/>
+      <c r="AF54" s="15" t="n"/>
+      <c r="AG54" s="15" t="n"/>
+      <c r="AH54" s="15" t="n"/>
+      <c r="AI54" s="15" t="n"/>
+      <c r="AJ54" s="15" t="n"/>
+      <c r="AK54" s="15" t="n"/>
+      <c r="AL54" s="15" t="n"/>
+      <c r="AM54" s="15" t="n"/>
+      <c r="AV54" s="15" t="n"/>
+      <c r="AW54" s="28" t="n"/>
+      <c r="AX54" s="15" t="n"/>
+      <c r="AY54" s="15" t="n"/>
+      <c r="AZ54" s="15" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n"/>
+      <c r="B55" s="15" t="n"/>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="16" t="n"/>
+      <c r="F55" s="15" t="n"/>
+      <c r="G55" s="15" t="n"/>
+      <c r="H55" s="15" t="n"/>
+      <c r="I55" s="15" t="n"/>
+      <c r="J55" s="15" t="n"/>
+      <c r="K55" s="15" t="n"/>
+      <c r="L55" s="15" t="n"/>
+      <c r="M55" s="15" t="n"/>
+      <c r="N55" s="15" t="n"/>
+      <c r="O55" s="15" t="n"/>
+      <c r="P55" s="15" t="n"/>
+      <c r="Q55" s="15" t="n"/>
+      <c r="R55" s="15" t="n"/>
+      <c r="S55" s="15" t="n"/>
+      <c r="T55" s="15" t="n"/>
+      <c r="U55" s="15" t="n"/>
+      <c r="V55" s="15" t="n"/>
+      <c r="W55" s="15" t="n"/>
+      <c r="X55" s="15" t="n"/>
+      <c r="Y55" s="15" t="n"/>
+      <c r="Z55" s="15" t="n"/>
+      <c r="AA55" s="15" t="n"/>
+      <c r="AB55" s="15" t="n"/>
+      <c r="AC55" s="15" t="n"/>
+      <c r="AD55" s="15" t="n"/>
+      <c r="AE55" s="15" t="n"/>
+      <c r="AF55" s="15" t="n"/>
+      <c r="AG55" s="15" t="n"/>
+      <c r="AH55" s="15" t="n"/>
+      <c r="AI55" s="15" t="n"/>
+      <c r="AJ55" s="15" t="n"/>
+      <c r="AK55" s="15" t="n"/>
+      <c r="AL55" s="15" t="n"/>
+      <c r="AM55" s="15" t="n"/>
+      <c r="AV55" s="15" t="n"/>
+      <c r="AW55" s="28" t="n"/>
+      <c r="AX55" s="15" t="n"/>
+      <c r="AY55" s="15" t="n"/>
+      <c r="AZ55" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -23016,7 +23211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR52"/>
+  <dimension ref="A1:AZ52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="34.83203125" customWidth="1" style="2" min="1" max="1"/>
@@ -23229,13 +23424,13 @@
       <c r="AK15" s="20" t="n"/>
       <c r="AL15" s="20" t="n"/>
       <c r="AM15" s="21" t="n"/>
-      <c r="AP15" s="19" t="inlineStr">
+      <c r="AX15" s="19" t="inlineStr">
         <is>
           <t>Custom Properties</t>
         </is>
       </c>
-      <c r="AQ15" s="20" t="n"/>
-      <c r="AR15" s="20" t="n"/>
+      <c r="AY15" s="20" t="n"/>
+      <c r="AZ15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -23433,19 +23628,59 @@
           <t>Pattern</t>
         </is>
       </c>
-      <c r="AN16" s="10" t="inlineStr">
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>Element Type</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Distance Metric</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Normalized</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>Embedding Model</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>Embedding Model Version</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Default Timezone</t>
+        </is>
+      </c>
+      <c r="AV16" s="10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="AO16" s="10" t="inlineStr">
+      <c r="AW16" s="10" t="inlineStr">
         <is>
           <t>Comments (internal)</t>
         </is>
       </c>
-      <c r="AP16" s="10" t="n"/>
-      <c r="AQ16" s="10" t="n"/>
-      <c r="AR16" s="10" t="n"/>
+      <c r="AX16" s="10" t="n"/>
+      <c r="AY16" s="10" t="n"/>
+      <c r="AZ16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -23503,15 +23738,15 @@
       <c r="AK17" s="15" t="n"/>
       <c r="AL17" s="15" t="n"/>
       <c r="AM17" s="15" t="n"/>
-      <c r="AN17" s="15" t="inlineStr">
+      <c r="AV17" s="15" t="inlineStr">
         <is>
           <t>archiveShipmentId</t>
         </is>
       </c>
-      <c r="AO17" s="28" t="n"/>
-      <c r="AP17" s="15" t="n"/>
-      <c r="AQ17" s="15" t="n"/>
-      <c r="AR17" s="15" t="n"/>
+      <c r="AW17" s="28" t="n"/>
+      <c r="AX17" s="15" t="n"/>
+      <c r="AY17" s="15" t="n"/>
+      <c r="AZ17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -23565,15 +23800,15 @@
       <c r="AK18" s="15" t="n"/>
       <c r="AL18" s="15" t="n"/>
       <c r="AM18" s="15" t="n"/>
-      <c r="AN18" s="15" t="inlineStr">
+      <c r="AV18" s="15" t="inlineStr">
         <is>
           <t>archiveArchivedAt</t>
         </is>
       </c>
-      <c r="AO18" s="28" t="n"/>
-      <c r="AP18" s="15" t="n"/>
-      <c r="AQ18" s="15" t="n"/>
-      <c r="AR18" s="15" t="n"/>
+      <c r="AW18" s="28" t="n"/>
+      <c r="AX18" s="15" t="n"/>
+      <c r="AY18" s="15" t="n"/>
+      <c r="AZ18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="17" t="n"/>
@@ -23615,11 +23850,11 @@
       <c r="AK19" s="15" t="n"/>
       <c r="AL19" s="15" t="n"/>
       <c r="AM19" s="15" t="n"/>
-      <c r="AN19" s="15" t="n"/>
-      <c r="AO19" s="28" t="n"/>
-      <c r="AP19" s="15" t="n"/>
-      <c r="AQ19" s="15" t="n"/>
-      <c r="AR19" s="15" t="n"/>
+      <c r="AV19" s="15" t="n"/>
+      <c r="AW19" s="28" t="n"/>
+      <c r="AX19" s="15" t="n"/>
+      <c r="AY19" s="15" t="n"/>
+      <c r="AZ19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="17" t="n"/>
@@ -23661,11 +23896,11 @@
       <c r="AK20" s="15" t="n"/>
       <c r="AL20" s="15" t="n"/>
       <c r="AM20" s="15" t="n"/>
-      <c r="AN20" s="15" t="n"/>
-      <c r="AO20" s="28" t="n"/>
-      <c r="AP20" s="15" t="n"/>
-      <c r="AQ20" s="15" t="n"/>
-      <c r="AR20" s="15" t="n"/>
+      <c r="AV20" s="15" t="n"/>
+      <c r="AW20" s="28" t="n"/>
+      <c r="AX20" s="15" t="n"/>
+      <c r="AY20" s="15" t="n"/>
+      <c r="AZ20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="17" t="n"/>
@@ -23707,11 +23942,11 @@
       <c r="AK21" s="15" t="n"/>
       <c r="AL21" s="15" t="n"/>
       <c r="AM21" s="15" t="n"/>
-      <c r="AN21" s="15" t="n"/>
-      <c r="AO21" s="28" t="n"/>
-      <c r="AP21" s="15" t="n"/>
-      <c r="AQ21" s="15" t="n"/>
-      <c r="AR21" s="15" t="n"/>
+      <c r="AV21" s="15" t="n"/>
+      <c r="AW21" s="28" t="n"/>
+      <c r="AX21" s="15" t="n"/>
+      <c r="AY21" s="15" t="n"/>
+      <c r="AZ21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="17" t="n"/>
@@ -23753,11 +23988,11 @@
       <c r="AK22" s="15" t="n"/>
       <c r="AL22" s="15" t="n"/>
       <c r="AM22" s="15" t="n"/>
-      <c r="AN22" s="15" t="n"/>
-      <c r="AO22" s="28" t="n"/>
-      <c r="AP22" s="15" t="n"/>
-      <c r="AQ22" s="15" t="n"/>
-      <c r="AR22" s="15" t="n"/>
+      <c r="AV22" s="15" t="n"/>
+      <c r="AW22" s="28" t="n"/>
+      <c r="AX22" s="15" t="n"/>
+      <c r="AY22" s="15" t="n"/>
+      <c r="AZ22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="17" t="n"/>
@@ -23799,11 +24034,11 @@
       <c r="AK23" s="15" t="n"/>
       <c r="AL23" s="15" t="n"/>
       <c r="AM23" s="15" t="n"/>
-      <c r="AN23" s="15" t="n"/>
-      <c r="AO23" s="28" t="n"/>
-      <c r="AP23" s="15" t="n"/>
-      <c r="AQ23" s="15" t="n"/>
-      <c r="AR23" s="15" t="n"/>
+      <c r="AV23" s="15" t="n"/>
+      <c r="AW23" s="28" t="n"/>
+      <c r="AX23" s="15" t="n"/>
+      <c r="AY23" s="15" t="n"/>
+      <c r="AZ23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="18" t="n"/>
@@ -23845,11 +24080,11 @@
       <c r="AK24" s="15" t="n"/>
       <c r="AL24" s="15" t="n"/>
       <c r="AM24" s="15" t="n"/>
-      <c r="AN24" s="15" t="n"/>
-      <c r="AO24" s="28" t="n"/>
-      <c r="AP24" s="15" t="n"/>
-      <c r="AQ24" s="15" t="n"/>
-      <c r="AR24" s="15" t="n"/>
+      <c r="AV24" s="15" t="n"/>
+      <c r="AW24" s="28" t="n"/>
+      <c r="AX24" s="15" t="n"/>
+      <c r="AY24" s="15" t="n"/>
+      <c r="AZ24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="18" t="n"/>
@@ -23891,11 +24126,11 @@
       <c r="AK25" s="15" t="n"/>
       <c r="AL25" s="15" t="n"/>
       <c r="AM25" s="15" t="n"/>
-      <c r="AN25" s="15" t="n"/>
-      <c r="AO25" s="28" t="n"/>
-      <c r="AP25" s="15" t="n"/>
-      <c r="AQ25" s="15" t="n"/>
-      <c r="AR25" s="15" t="n"/>
+      <c r="AV25" s="15" t="n"/>
+      <c r="AW25" s="28" t="n"/>
+      <c r="AX25" s="15" t="n"/>
+      <c r="AY25" s="15" t="n"/>
+      <c r="AZ25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="18" t="n"/>
@@ -23937,11 +24172,11 @@
       <c r="AK26" s="15" t="n"/>
       <c r="AL26" s="15" t="n"/>
       <c r="AM26" s="15" t="n"/>
-      <c r="AN26" s="15" t="n"/>
-      <c r="AO26" s="28" t="n"/>
-      <c r="AP26" s="15" t="n"/>
-      <c r="AQ26" s="15" t="n"/>
-      <c r="AR26" s="15" t="n"/>
+      <c r="AV26" s="15" t="n"/>
+      <c r="AW26" s="28" t="n"/>
+      <c r="AX26" s="15" t="n"/>
+      <c r="AY26" s="15" t="n"/>
+      <c r="AZ26" s="15" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="17" t="n"/>
@@ -23983,11 +24218,11 @@
       <c r="AK27" s="15" t="n"/>
       <c r="AL27" s="15" t="n"/>
       <c r="AM27" s="15" t="n"/>
-      <c r="AN27" s="15" t="n"/>
-      <c r="AO27" s="28" t="n"/>
-      <c r="AP27" s="15" t="n"/>
-      <c r="AQ27" s="15" t="n"/>
-      <c r="AR27" s="15" t="n"/>
+      <c r="AV27" s="15" t="n"/>
+      <c r="AW27" s="28" t="n"/>
+      <c r="AX27" s="15" t="n"/>
+      <c r="AY27" s="15" t="n"/>
+      <c r="AZ27" s="15" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="17" t="n"/>
@@ -24029,11 +24264,11 @@
       <c r="AK28" s="15" t="n"/>
       <c r="AL28" s="15" t="n"/>
       <c r="AM28" s="15" t="n"/>
-      <c r="AN28" s="15" t="n"/>
-      <c r="AO28" s="28" t="n"/>
-      <c r="AP28" s="15" t="n"/>
-      <c r="AQ28" s="15" t="n"/>
-      <c r="AR28" s="15" t="n"/>
+      <c r="AV28" s="15" t="n"/>
+      <c r="AW28" s="28" t="n"/>
+      <c r="AX28" s="15" t="n"/>
+      <c r="AY28" s="15" t="n"/>
+      <c r="AZ28" s="15" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="17" t="n"/>
@@ -24075,11 +24310,11 @@
       <c r="AK29" s="15" t="n"/>
       <c r="AL29" s="15" t="n"/>
       <c r="AM29" s="15" t="n"/>
-      <c r="AN29" s="15" t="n"/>
-      <c r="AO29" s="28" t="n"/>
-      <c r="AP29" s="15" t="n"/>
-      <c r="AQ29" s="15" t="n"/>
-      <c r="AR29" s="15" t="n"/>
+      <c r="AV29" s="15" t="n"/>
+      <c r="AW29" s="28" t="n"/>
+      <c r="AX29" s="15" t="n"/>
+      <c r="AY29" s="15" t="n"/>
+      <c r="AZ29" s="15" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="17" t="n"/>
@@ -24121,11 +24356,11 @@
       <c r="AK30" s="15" t="n"/>
       <c r="AL30" s="15" t="n"/>
       <c r="AM30" s="15" t="n"/>
-      <c r="AN30" s="15" t="n"/>
-      <c r="AO30" s="28" t="n"/>
-      <c r="AP30" s="15" t="n"/>
-      <c r="AQ30" s="15" t="n"/>
-      <c r="AR30" s="15" t="n"/>
+      <c r="AV30" s="15" t="n"/>
+      <c r="AW30" s="28" t="n"/>
+      <c r="AX30" s="15" t="n"/>
+      <c r="AY30" s="15" t="n"/>
+      <c r="AZ30" s="15" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="n"/>
@@ -24167,11 +24402,11 @@
       <c r="AK31" s="15" t="n"/>
       <c r="AL31" s="15" t="n"/>
       <c r="AM31" s="15" t="n"/>
-      <c r="AN31" s="15" t="n"/>
-      <c r="AO31" s="28" t="n"/>
-      <c r="AP31" s="15" t="n"/>
-      <c r="AQ31" s="15" t="n"/>
-      <c r="AR31" s="15" t="n"/>
+      <c r="AV31" s="15" t="n"/>
+      <c r="AW31" s="28" t="n"/>
+      <c r="AX31" s="15" t="n"/>
+      <c r="AY31" s="15" t="n"/>
+      <c r="AZ31" s="15" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="17" t="n"/>
@@ -24213,11 +24448,11 @@
       <c r="AK32" s="15" t="n"/>
       <c r="AL32" s="15" t="n"/>
       <c r="AM32" s="15" t="n"/>
-      <c r="AN32" s="15" t="n"/>
-      <c r="AO32" s="28" t="n"/>
-      <c r="AP32" s="15" t="n"/>
-      <c r="AQ32" s="15" t="n"/>
-      <c r="AR32" s="15" t="n"/>
+      <c r="AV32" s="15" t="n"/>
+      <c r="AW32" s="28" t="n"/>
+      <c r="AX32" s="15" t="n"/>
+      <c r="AY32" s="15" t="n"/>
+      <c r="AZ32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="n"/>
@@ -24259,11 +24494,11 @@
       <c r="AK33" s="15" t="n"/>
       <c r="AL33" s="15" t="n"/>
       <c r="AM33" s="15" t="n"/>
-      <c r="AN33" s="15" t="n"/>
-      <c r="AO33" s="28" t="n"/>
-      <c r="AP33" s="15" t="n"/>
-      <c r="AQ33" s="15" t="n"/>
-      <c r="AR33" s="15" t="n"/>
+      <c r="AV33" s="15" t="n"/>
+      <c r="AW33" s="28" t="n"/>
+      <c r="AX33" s="15" t="n"/>
+      <c r="AY33" s="15" t="n"/>
+      <c r="AZ33" s="15" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="17" t="n"/>
@@ -24305,11 +24540,11 @@
       <c r="AK34" s="15" t="n"/>
       <c r="AL34" s="15" t="n"/>
       <c r="AM34" s="15" t="n"/>
-      <c r="AN34" s="15" t="n"/>
-      <c r="AO34" s="28" t="n"/>
-      <c r="AP34" s="15" t="n"/>
-      <c r="AQ34" s="15" t="n"/>
-      <c r="AR34" s="15" t="n"/>
+      <c r="AV34" s="15" t="n"/>
+      <c r="AW34" s="28" t="n"/>
+      <c r="AX34" s="15" t="n"/>
+      <c r="AY34" s="15" t="n"/>
+      <c r="AZ34" s="15" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="17" t="n"/>
@@ -24351,11 +24586,11 @@
       <c r="AK35" s="15" t="n"/>
       <c r="AL35" s="15" t="n"/>
       <c r="AM35" s="15" t="n"/>
-      <c r="AN35" s="15" t="n"/>
-      <c r="AO35" s="28" t="n"/>
-      <c r="AP35" s="15" t="n"/>
-      <c r="AQ35" s="15" t="n"/>
-      <c r="AR35" s="15" t="n"/>
+      <c r="AV35" s="15" t="n"/>
+      <c r="AW35" s="28" t="n"/>
+      <c r="AX35" s="15" t="n"/>
+      <c r="AY35" s="15" t="n"/>
+      <c r="AZ35" s="15" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="17" t="n"/>
@@ -24397,11 +24632,11 @@
       <c r="AK36" s="15" t="n"/>
       <c r="AL36" s="15" t="n"/>
       <c r="AM36" s="15" t="n"/>
-      <c r="AN36" s="15" t="n"/>
-      <c r="AO36" s="28" t="n"/>
-      <c r="AP36" s="15" t="n"/>
-      <c r="AQ36" s="15" t="n"/>
-      <c r="AR36" s="15" t="n"/>
+      <c r="AV36" s="15" t="n"/>
+      <c r="AW36" s="28" t="n"/>
+      <c r="AX36" s="15" t="n"/>
+      <c r="AY36" s="15" t="n"/>
+      <c r="AZ36" s="15" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="17" t="n"/>
@@ -24443,11 +24678,11 @@
       <c r="AK37" s="15" t="n"/>
       <c r="AL37" s="15" t="n"/>
       <c r="AM37" s="15" t="n"/>
-      <c r="AN37" s="15" t="n"/>
-      <c r="AO37" s="28" t="n"/>
-      <c r="AP37" s="15" t="n"/>
-      <c r="AQ37" s="15" t="n"/>
-      <c r="AR37" s="15" t="n"/>
+      <c r="AV37" s="15" t="n"/>
+      <c r="AW37" s="28" t="n"/>
+      <c r="AX37" s="15" t="n"/>
+      <c r="AY37" s="15" t="n"/>
+      <c r="AZ37" s="15" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="17" t="n"/>
@@ -24489,11 +24724,11 @@
       <c r="AK38" s="15" t="n"/>
       <c r="AL38" s="15" t="n"/>
       <c r="AM38" s="15" t="n"/>
-      <c r="AN38" s="15" t="n"/>
-      <c r="AO38" s="28" t="n"/>
-      <c r="AP38" s="15" t="n"/>
-      <c r="AQ38" s="15" t="n"/>
-      <c r="AR38" s="15" t="n"/>
+      <c r="AV38" s="15" t="n"/>
+      <c r="AW38" s="28" t="n"/>
+      <c r="AX38" s="15" t="n"/>
+      <c r="AY38" s="15" t="n"/>
+      <c r="AZ38" s="15" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="17" t="n"/>
@@ -24535,11 +24770,11 @@
       <c r="AK39" s="15" t="n"/>
       <c r="AL39" s="15" t="n"/>
       <c r="AM39" s="15" t="n"/>
-      <c r="AN39" s="15" t="n"/>
-      <c r="AO39" s="28" t="n"/>
-      <c r="AP39" s="15" t="n"/>
-      <c r="AQ39" s="15" t="n"/>
-      <c r="AR39" s="15" t="n"/>
+      <c r="AV39" s="15" t="n"/>
+      <c r="AW39" s="28" t="n"/>
+      <c r="AX39" s="15" t="n"/>
+      <c r="AY39" s="15" t="n"/>
+      <c r="AZ39" s="15" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="17" t="n"/>
@@ -24581,11 +24816,11 @@
       <c r="AK40" s="15" t="n"/>
       <c r="AL40" s="15" t="n"/>
       <c r="AM40" s="15" t="n"/>
-      <c r="AN40" s="15" t="n"/>
-      <c r="AO40" s="28" t="n"/>
-      <c r="AP40" s="15" t="n"/>
-      <c r="AQ40" s="15" t="n"/>
-      <c r="AR40" s="15" t="n"/>
+      <c r="AV40" s="15" t="n"/>
+      <c r="AW40" s="28" t="n"/>
+      <c r="AX40" s="15" t="n"/>
+      <c r="AY40" s="15" t="n"/>
+      <c r="AZ40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="17" t="n"/>
@@ -24627,11 +24862,11 @@
       <c r="AK41" s="15" t="n"/>
       <c r="AL41" s="15" t="n"/>
       <c r="AM41" s="15" t="n"/>
-      <c r="AN41" s="15" t="n"/>
-      <c r="AO41" s="28" t="n"/>
-      <c r="AP41" s="15" t="n"/>
-      <c r="AQ41" s="15" t="n"/>
-      <c r="AR41" s="15" t="n"/>
+      <c r="AV41" s="15" t="n"/>
+      <c r="AW41" s="28" t="n"/>
+      <c r="AX41" s="15" t="n"/>
+      <c r="AY41" s="15" t="n"/>
+      <c r="AZ41" s="15" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="17" t="n"/>
@@ -24673,11 +24908,11 @@
       <c r="AK42" s="15" t="n"/>
       <c r="AL42" s="15" t="n"/>
       <c r="AM42" s="15" t="n"/>
-      <c r="AN42" s="15" t="n"/>
-      <c r="AO42" s="28" t="n"/>
-      <c r="AP42" s="15" t="n"/>
-      <c r="AQ42" s="15" t="n"/>
-      <c r="AR42" s="15" t="n"/>
+      <c r="AV42" s="15" t="n"/>
+      <c r="AW42" s="28" t="n"/>
+      <c r="AX42" s="15" t="n"/>
+      <c r="AY42" s="15" t="n"/>
+      <c r="AZ42" s="15" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="n"/>
@@ -24719,11 +24954,11 @@
       <c r="AK43" s="15" t="n"/>
       <c r="AL43" s="15" t="n"/>
       <c r="AM43" s="15" t="n"/>
-      <c r="AN43" s="15" t="n"/>
-      <c r="AO43" s="28" t="n"/>
-      <c r="AP43" s="15" t="n"/>
-      <c r="AQ43" s="15" t="n"/>
-      <c r="AR43" s="15" t="n"/>
+      <c r="AV43" s="15" t="n"/>
+      <c r="AW43" s="28" t="n"/>
+      <c r="AX43" s="15" t="n"/>
+      <c r="AY43" s="15" t="n"/>
+      <c r="AZ43" s="15" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="17" t="n"/>
@@ -24765,11 +25000,11 @@
       <c r="AK44" s="15" t="n"/>
       <c r="AL44" s="15" t="n"/>
       <c r="AM44" s="15" t="n"/>
-      <c r="AN44" s="15" t="n"/>
-      <c r="AO44" s="28" t="n"/>
-      <c r="AP44" s="15" t="n"/>
-      <c r="AQ44" s="15" t="n"/>
-      <c r="AR44" s="15" t="n"/>
+      <c r="AV44" s="15" t="n"/>
+      <c r="AW44" s="28" t="n"/>
+      <c r="AX44" s="15" t="n"/>
+      <c r="AY44" s="15" t="n"/>
+      <c r="AZ44" s="15" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n"/>
@@ -24811,11 +25046,11 @@
       <c r="AK45" s="15" t="n"/>
       <c r="AL45" s="15" t="n"/>
       <c r="AM45" s="15" t="n"/>
-      <c r="AN45" s="15" t="n"/>
-      <c r="AO45" s="28" t="n"/>
-      <c r="AP45" s="15" t="n"/>
-      <c r="AQ45" s="15" t="n"/>
-      <c r="AR45" s="15" t="n"/>
+      <c r="AV45" s="15" t="n"/>
+      <c r="AW45" s="28" t="n"/>
+      <c r="AX45" s="15" t="n"/>
+      <c r="AY45" s="15" t="n"/>
+      <c r="AZ45" s="15" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="17" t="n"/>
@@ -24857,11 +25092,11 @@
       <c r="AK46" s="15" t="n"/>
       <c r="AL46" s="15" t="n"/>
       <c r="AM46" s="15" t="n"/>
-      <c r="AN46" s="15" t="n"/>
-      <c r="AO46" s="28" t="n"/>
-      <c r="AP46" s="15" t="n"/>
-      <c r="AQ46" s="15" t="n"/>
-      <c r="AR46" s="15" t="n"/>
+      <c r="AV46" s="15" t="n"/>
+      <c r="AW46" s="28" t="n"/>
+      <c r="AX46" s="15" t="n"/>
+      <c r="AY46" s="15" t="n"/>
+      <c r="AZ46" s="15" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="17" t="n"/>
@@ -24903,11 +25138,11 @@
       <c r="AK47" s="15" t="n"/>
       <c r="AL47" s="15" t="n"/>
       <c r="AM47" s="15" t="n"/>
-      <c r="AN47" s="15" t="n"/>
-      <c r="AO47" s="28" t="n"/>
-      <c r="AP47" s="15" t="n"/>
-      <c r="AQ47" s="15" t="n"/>
-      <c r="AR47" s="15" t="n"/>
+      <c r="AV47" s="15" t="n"/>
+      <c r="AW47" s="28" t="n"/>
+      <c r="AX47" s="15" t="n"/>
+      <c r="AY47" s="15" t="n"/>
+      <c r="AZ47" s="15" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="17" t="n"/>
@@ -24949,11 +25184,11 @@
       <c r="AK48" s="15" t="n"/>
       <c r="AL48" s="15" t="n"/>
       <c r="AM48" s="15" t="n"/>
-      <c r="AN48" s="15" t="n"/>
-      <c r="AO48" s="28" t="n"/>
-      <c r="AP48" s="15" t="n"/>
-      <c r="AQ48" s="15" t="n"/>
-      <c r="AR48" s="15" t="n"/>
+      <c r="AV48" s="15" t="n"/>
+      <c r="AW48" s="28" t="n"/>
+      <c r="AX48" s="15" t="n"/>
+      <c r="AY48" s="15" t="n"/>
+      <c r="AZ48" s="15" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n"/>
@@ -24995,11 +25230,11 @@
       <c r="AK49" s="15" t="n"/>
       <c r="AL49" s="15" t="n"/>
       <c r="AM49" s="15" t="n"/>
-      <c r="AN49" s="15" t="n"/>
-      <c r="AO49" s="28" t="n"/>
-      <c r="AP49" s="15" t="n"/>
-      <c r="AQ49" s="15" t="n"/>
-      <c r="AR49" s="15" t="n"/>
+      <c r="AV49" s="15" t="n"/>
+      <c r="AW49" s="28" t="n"/>
+      <c r="AX49" s="15" t="n"/>
+      <c r="AY49" s="15" t="n"/>
+      <c r="AZ49" s="15" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="17" t="n"/>
@@ -25041,11 +25276,11 @@
       <c r="AK50" s="15" t="n"/>
       <c r="AL50" s="15" t="n"/>
       <c r="AM50" s="15" t="n"/>
-      <c r="AN50" s="15" t="n"/>
-      <c r="AO50" s="28" t="n"/>
-      <c r="AP50" s="15" t="n"/>
-      <c r="AQ50" s="15" t="n"/>
-      <c r="AR50" s="15" t="n"/>
+      <c r="AV50" s="15" t="n"/>
+      <c r="AW50" s="28" t="n"/>
+      <c r="AX50" s="15" t="n"/>
+      <c r="AY50" s="15" t="n"/>
+      <c r="AZ50" s="15" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="17" t="n"/>
@@ -25087,11 +25322,11 @@
       <c r="AK51" s="15" t="n"/>
       <c r="AL51" s="15" t="n"/>
       <c r="AM51" s="15" t="n"/>
-      <c r="AN51" s="15" t="n"/>
-      <c r="AO51" s="28" t="n"/>
-      <c r="AP51" s="15" t="n"/>
-      <c r="AQ51" s="15" t="n"/>
-      <c r="AR51" s="15" t="n"/>
+      <c r="AV51" s="15" t="n"/>
+      <c r="AW51" s="28" t="n"/>
+      <c r="AX51" s="15" t="n"/>
+      <c r="AY51" s="15" t="n"/>
+      <c r="AZ51" s="15" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="17" t="n"/>
@@ -25133,11 +25368,11 @@
       <c r="AK52" s="15" t="n"/>
       <c r="AL52" s="15" t="n"/>
       <c r="AM52" s="15" t="n"/>
-      <c r="AN52" s="15" t="n"/>
-      <c r="AO52" s="28" t="n"/>
-      <c r="AP52" s="15" t="n"/>
-      <c r="AQ52" s="15" t="n"/>
-      <c r="AR52" s="15" t="n"/>
+      <c r="AV52" s="15" t="n"/>
+      <c r="AW52" s="28" t="n"/>
+      <c r="AX52" s="15" t="n"/>
+      <c r="AY52" s="15" t="n"/>
+      <c r="AZ52" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -26861,7 +27096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="33.1640625" customWidth="1" style="2" min="1" max="1"/>
@@ -26942,13 +27177,13 @@
       <c r="A8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="I9" s="19" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>Custom Properties</t>
         </is>
       </c>
-      <c r="J9" s="20" t="n"/>
       <c r="K9" s="20" t="n"/>
+      <c r="L9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -26971,29 +27206,34 @@
           <t>Role</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Date In</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Date Out</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Replaced By Username</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="I10" s="10" t="n"/>
       <c r="J10" s="10" t="n"/>
       <c r="K10" s="10" t="n"/>
+      <c r="L10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
@@ -27016,21 +27256,26 @@
           <t>owner</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>oncall</t>
+        </is>
+      </c>
+      <c r="F11" s="36" t="inlineStr">
         <is>
           <t>2020-01-01</t>
         </is>
       </c>
-      <c r="F11" s="36" t="n"/>
       <c r="G11" s="36" t="n"/>
-      <c r="H11" s="36" t="inlineStr">
+      <c r="H11" s="36" t="n"/>
+      <c r="I11" s="36" t="inlineStr">
         <is>
           <t>memberJdoe</t>
         </is>
       </c>
-      <c r="I11" s="15" t="n"/>
       <c r="J11" s="15" t="n"/>
       <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
@@ -27049,220 +27294,220 @@
           <t>reader</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="F12" s="36" t="inlineStr">
         <is>
           <t>2021-06-01</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>2024-10-10</t>
         </is>
       </c>
-      <c r="G12" s="36" t="inlineStr">
+      <c r="H12" s="36" t="inlineStr">
         <is>
           <t>jdoe</t>
         </is>
       </c>
-      <c r="H12" s="36" t="n"/>
-      <c r="I12" s="15" t="n"/>
+      <c r="I12" s="36" t="n"/>
       <c r="J12" s="15" t="n"/>
       <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="36" t="n"/>
       <c r="B13" s="36" t="n"/>
       <c r="C13" s="36" t="n"/>
       <c r="D13" s="36" t="n"/>
-      <c r="E13" s="36" t="n"/>
       <c r="F13" s="36" t="n"/>
       <c r="G13" s="36" t="n"/>
       <c r="H13" s="36" t="n"/>
-      <c r="I13" s="15" t="n"/>
+      <c r="I13" s="36" t="n"/>
       <c r="J13" s="15" t="n"/>
       <c r="K13" s="15" t="n"/>
+      <c r="L13" s="15" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="36" t="n"/>
       <c r="B14" s="36" t="n"/>
       <c r="C14" s="36" t="n"/>
       <c r="D14" s="36" t="n"/>
-      <c r="E14" s="36" t="n"/>
       <c r="F14" s="36" t="n"/>
       <c r="G14" s="36" t="n"/>
       <c r="H14" s="36" t="n"/>
-      <c r="I14" s="15" t="n"/>
+      <c r="I14" s="36" t="n"/>
       <c r="J14" s="15" t="n"/>
       <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="36" t="n"/>
       <c r="B15" s="36" t="n"/>
       <c r="C15" s="36" t="n"/>
       <c r="D15" s="36" t="n"/>
-      <c r="E15" s="36" t="n"/>
       <c r="F15" s="36" t="n"/>
       <c r="G15" s="36" t="n"/>
       <c r="H15" s="36" t="n"/>
-      <c r="I15" s="15" t="n"/>
+      <c r="I15" s="36" t="n"/>
       <c r="J15" s="15" t="n"/>
       <c r="K15" s="15" t="n"/>
+      <c r="L15" s="15" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="36" t="n"/>
       <c r="B16" s="36" t="n"/>
       <c r="C16" s="36" t="n"/>
       <c r="D16" s="36" t="n"/>
-      <c r="E16" s="36" t="n"/>
       <c r="F16" s="36" t="n"/>
       <c r="G16" s="36" t="n"/>
       <c r="H16" s="36" t="n"/>
-      <c r="I16" s="15" t="n"/>
+      <c r="I16" s="36" t="n"/>
       <c r="J16" s="15" t="n"/>
       <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="36" t="n"/>
       <c r="B17" s="36" t="n"/>
       <c r="C17" s="36" t="n"/>
       <c r="D17" s="36" t="n"/>
-      <c r="E17" s="36" t="n"/>
       <c r="F17" s="36" t="n"/>
       <c r="G17" s="36" t="n"/>
       <c r="H17" s="36" t="n"/>
-      <c r="I17" s="15" t="n"/>
+      <c r="I17" s="36" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="15" t="n"/>
+      <c r="L17" s="15" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="36" t="n"/>
       <c r="B18" s="36" t="n"/>
       <c r="C18" s="36" t="n"/>
       <c r="D18" s="36" t="n"/>
-      <c r="E18" s="36" t="n"/>
       <c r="F18" s="36" t="n"/>
       <c r="G18" s="36" t="n"/>
       <c r="H18" s="36" t="n"/>
-      <c r="I18" s="15" t="n"/>
+      <c r="I18" s="36" t="n"/>
       <c r="J18" s="15" t="n"/>
       <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="36" t="n"/>
       <c r="B19" s="36" t="n"/>
       <c r="C19" s="36" t="n"/>
       <c r="D19" s="36" t="n"/>
-      <c r="E19" s="36" t="n"/>
       <c r="F19" s="36" t="n"/>
       <c r="G19" s="36" t="n"/>
       <c r="H19" s="36" t="n"/>
-      <c r="I19" s="15" t="n"/>
+      <c r="I19" s="36" t="n"/>
       <c r="J19" s="15" t="n"/>
       <c r="K19" s="15" t="n"/>
+      <c r="L19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="36" t="n"/>
       <c r="B20" s="36" t="n"/>
       <c r="C20" s="36" t="n"/>
       <c r="D20" s="36" t="n"/>
-      <c r="E20" s="36" t="n"/>
       <c r="F20" s="36" t="n"/>
       <c r="G20" s="36" t="n"/>
       <c r="H20" s="36" t="n"/>
-      <c r="I20" s="15" t="n"/>
+      <c r="I20" s="36" t="n"/>
       <c r="J20" s="15" t="n"/>
       <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="36" t="n"/>
       <c r="B21" s="36" t="n"/>
       <c r="C21" s="36" t="n"/>
       <c r="D21" s="36" t="n"/>
-      <c r="E21" s="36" t="n"/>
       <c r="F21" s="36" t="n"/>
       <c r="G21" s="36" t="n"/>
       <c r="H21" s="36" t="n"/>
-      <c r="I21" s="15" t="n"/>
+      <c r="I21" s="36" t="n"/>
       <c r="J21" s="15" t="n"/>
       <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="36" t="n"/>
       <c r="B22" s="36" t="n"/>
       <c r="C22" s="36" t="n"/>
       <c r="D22" s="36" t="n"/>
-      <c r="E22" s="36" t="n"/>
       <c r="F22" s="36" t="n"/>
       <c r="G22" s="36" t="n"/>
       <c r="H22" s="36" t="n"/>
-      <c r="I22" s="15" t="n"/>
+      <c r="I22" s="36" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="36" t="n"/>
       <c r="B23" s="36" t="n"/>
       <c r="C23" s="36" t="n"/>
       <c r="D23" s="36" t="n"/>
-      <c r="E23" s="36" t="n"/>
       <c r="F23" s="36" t="n"/>
       <c r="G23" s="36" t="n"/>
       <c r="H23" s="36" t="n"/>
-      <c r="I23" s="15" t="n"/>
+      <c r="I23" s="36" t="n"/>
       <c r="J23" s="15" t="n"/>
       <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="36" t="n"/>
       <c r="B24" s="36" t="n"/>
       <c r="C24" s="36" t="n"/>
       <c r="D24" s="36" t="n"/>
-      <c r="E24" s="36" t="n"/>
       <c r="F24" s="36" t="n"/>
       <c r="G24" s="36" t="n"/>
       <c r="H24" s="36" t="n"/>
-      <c r="I24" s="15" t="n"/>
+      <c r="I24" s="36" t="n"/>
       <c r="J24" s="15" t="n"/>
       <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="36" t="n"/>
       <c r="B25" s="36" t="n"/>
       <c r="C25" s="36" t="n"/>
       <c r="D25" s="36" t="n"/>
-      <c r="E25" s="36" t="n"/>
       <c r="F25" s="36" t="n"/>
       <c r="G25" s="36" t="n"/>
       <c r="H25" s="36" t="n"/>
-      <c r="I25" s="15" t="n"/>
+      <c r="I25" s="36" t="n"/>
       <c r="J25" s="15" t="n"/>
       <c r="K25" s="15" t="n"/>
+      <c r="L25" s="15" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="36" t="n"/>
       <c r="B26" s="36" t="n"/>
       <c r="C26" s="36" t="n"/>
       <c r="D26" s="36" t="n"/>
-      <c r="E26" s="36" t="n"/>
       <c r="F26" s="36" t="n"/>
       <c r="G26" s="36" t="n"/>
       <c r="H26" s="36" t="n"/>
-      <c r="I26" s="15" t="n"/>
+      <c r="I26" s="36" t="n"/>
       <c r="J26" s="15" t="n"/>
       <c r="K26" s="15" t="n"/>
+      <c r="L26" s="15" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="36" t="n"/>
       <c r="B27" s="36" t="n"/>
       <c r="C27" s="36" t="n"/>
       <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
       <c r="F27" s="36" t="n"/>
       <c r="G27" s="36" t="n"/>
       <c r="H27" s="36" t="n"/>
-      <c r="I27" s="15" t="n"/>
+      <c r="I27" s="36" t="n"/>
       <c r="J27" s="15" t="n"/>
       <c r="K27" s="15" t="n"/>
+      <c r="L27" s="15" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>